<commit_message>
Okno serwisowe 21.04.2026 - aktualizacja EXCEL
</commit_message>
<xml_diff>
--- a/assets/excel/en/national_sdg_indicators.xlsx
+++ b/assets/excel/en/national_sdg_indicators.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sidwab\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dregerj\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2EF6D31-E2C5-4043-AECF-C8E48B344757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53329364-CB59-4AEB-9E58-5C0F53FED924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2090" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2090" uniqueCount="413">
   <si>
     <t>sdg.gov.pl/en</t>
   </si>
@@ -1240,6 +1240,9 @@
     <t>17.4.a Participation of National Revenue Administration in twinning projects, activities financed from Taiex and from domestic resources</t>
   </si>
   <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>Ministry of Finance</t>
   </si>
   <si>
@@ -1264,7 +1267,7 @@
     <t>The Ministry of Economic Development and Technology / The Chancellery of the  Prime Minister</t>
   </si>
   <si>
-    <t>Last update: 24-03-2026, 11:45</t>
+    <t>Last update: 21-04-2026, 11:39</t>
   </si>
 </sst>
 </file>
@@ -2087,7 +2090,7 @@
         <v>36</v>
       </c>
       <c r="U6" s="4">
-        <v>41.8</v>
+        <v>41.1</v>
       </c>
       <c r="V6" s="4">
         <v>44.2</v>
@@ -2154,7 +2157,7 @@
         <v>51.4</v>
       </c>
       <c r="U7" s="4">
-        <v>60.4</v>
+        <v>58.2</v>
       </c>
       <c r="V7" s="4">
         <v>60.5</v>
@@ -2221,7 +2224,7 @@
         <v>15.1</v>
       </c>
       <c r="U8" s="4">
-        <v>21</v>
+        <v>19.8</v>
       </c>
       <c r="V8" s="4">
         <v>23.5</v>
@@ -6216,7 +6219,9 @@
       <c r="U75" s="4">
         <v>95.4</v>
       </c>
-      <c r="V75" s="3"/>
+      <c r="V75" s="4">
+        <v>95.1</v>
+      </c>
       <c r="W75" s="2" t="s">
         <v>117</v>
       </c>
@@ -8968,7 +8973,7 @@
         <v>36</v>
       </c>
       <c r="U125" s="4">
-        <v>41.8</v>
+        <v>41.1</v>
       </c>
       <c r="V125" s="4">
         <v>44.2</v>
@@ -9035,7 +9040,7 @@
         <v>51.4</v>
       </c>
       <c r="U126" s="4">
-        <v>60.4</v>
+        <v>58.2</v>
       </c>
       <c r="V126" s="4">
         <v>60.5</v>
@@ -9102,7 +9107,7 @@
         <v>15.1</v>
       </c>
       <c r="U127" s="4">
-        <v>21</v>
+        <v>19.8</v>
       </c>
       <c r="V127" s="4">
         <v>23.5</v>
@@ -13269,7 +13274,9 @@
       <c r="U188" s="4">
         <v>15.2</v>
       </c>
-      <c r="V188" s="3"/>
+      <c r="V188" s="4">
+        <v>15.9</v>
+      </c>
       <c r="W188" s="2" t="s">
         <v>30</v>
       </c>
@@ -14171,7 +14178,9 @@
       <c r="U204" s="6">
         <v>294</v>
       </c>
-      <c r="V204" s="3"/>
+      <c r="V204" s="6">
+        <v>372</v>
+      </c>
       <c r="W204" s="2" t="s">
         <v>258</v>
       </c>
@@ -16197,7 +16206,7 @@
         <v>95</v>
       </c>
       <c r="Q236" s="4">
-        <v>90.5</v>
+        <v>90.4</v>
       </c>
       <c r="R236" s="4">
         <v>99</v>
@@ -16206,9 +16215,11 @@
         <v>94.2</v>
       </c>
       <c r="T236" s="4">
-        <v>84.8</v>
-      </c>
-      <c r="U236" s="3"/>
+        <v>84.9</v>
+      </c>
+      <c r="U236" s="4">
+        <v>83.4</v>
+      </c>
       <c r="V236" s="3"/>
       <c r="W236" s="2" t="s">
         <v>313</v>
@@ -16237,45 +16248,47 @@
         <v>100</v>
       </c>
       <c r="H237" s="4">
-        <v>99.6</v>
+        <v>99.7</v>
       </c>
       <c r="I237" s="4">
         <v>97.8</v>
       </c>
       <c r="J237" s="4">
-        <v>96.8</v>
+        <v>96.7</v>
       </c>
       <c r="K237" s="4">
-        <v>93.7</v>
+        <v>93.6</v>
       </c>
       <c r="L237" s="4">
-        <v>94.4</v>
+        <v>94.3</v>
       </c>
       <c r="M237" s="4">
-        <v>97</v>
+        <v>96.9</v>
       </c>
       <c r="N237" s="4">
-        <v>100.6</v>
+        <v>100.5</v>
       </c>
       <c r="O237" s="4">
-        <v>100.6</v>
+        <v>100.4</v>
       </c>
       <c r="P237" s="4">
-        <v>95.1</v>
+        <v>94.9</v>
       </c>
       <c r="Q237" s="4">
-        <v>91.5</v>
+        <v>91.2</v>
       </c>
       <c r="R237" s="4">
-        <v>98.4</v>
+        <v>98.2</v>
       </c>
       <c r="S237" s="4">
-        <v>93.8</v>
+        <v>93.6</v>
       </c>
       <c r="T237" s="4">
-        <v>85.8</v>
-      </c>
-      <c r="U237" s="3"/>
+        <v>85.7</v>
+      </c>
+      <c r="U237" s="4">
+        <v>84.2</v>
+      </c>
       <c r="V237" s="3"/>
       <c r="W237" s="2" t="s">
         <v>313</v>
@@ -16483,7 +16496,9 @@
       <c r="U240" s="6">
         <v>33623</v>
       </c>
-      <c r="V240" s="3"/>
+      <c r="V240" s="6">
+        <v>37777</v>
+      </c>
       <c r="W240" s="2" t="s">
         <v>322</v>
       </c>
@@ -16997,7 +17012,9 @@
       <c r="U248" s="6">
         <v>80</v>
       </c>
-      <c r="V248" s="3"/>
+      <c r="V248" s="6">
+        <v>86</v>
+      </c>
       <c r="W248" s="2" t="s">
         <v>337</v>
       </c>
@@ -17091,7 +17108,9 @@
       <c r="U250" s="6">
         <v>44</v>
       </c>
-      <c r="V250" s="3"/>
+      <c r="V250" s="6">
+        <v>89</v>
+      </c>
       <c r="W250" s="2" t="s">
         <v>343</v>
       </c>
@@ -20017,7 +20036,7 @@
         <v>28</v>
       </c>
       <c r="F295" s="3" t="s">
-        <v>257</v>
+        <v>403</v>
       </c>
       <c r="G295" s="3"/>
       <c r="H295" s="3"/>
@@ -20054,7 +20073,7 @@
         <v>2</v>
       </c>
       <c r="W295" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="296" spans="1:23" ht="27" x14ac:dyDescent="0.25">
@@ -20062,10 +20081,10 @@
         <v>388</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D296" s="2" t="s">
         <v>27</v>
@@ -20074,7 +20093,7 @@
         <v>28</v>
       </c>
       <c r="F296" s="3" t="s">
-        <v>257</v>
+        <v>403</v>
       </c>
       <c r="G296" s="3"/>
       <c r="H296" s="3"/>
@@ -20121,7 +20140,7 @@
         <v>2</v>
       </c>
       <c r="W296" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="297" spans="1:23" ht="27" x14ac:dyDescent="0.25">
@@ -20129,10 +20148,10 @@
         <v>388</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D297" s="2" t="s">
         <v>27</v>
@@ -20184,7 +20203,7 @@
         <v>69</v>
       </c>
       <c r="W297" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="298" spans="1:23" ht="45" x14ac:dyDescent="0.25">
@@ -20192,10 +20211,10 @@
         <v>388</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D298" s="2" t="s">
         <v>27</v>
@@ -20229,13 +20248,13 @@
         <v>97</v>
       </c>
       <c r="W298" s="2" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="299" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="300" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A300" s="10" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B300" s="8"/>
     </row>
@@ -20250,7 +20269,7 @@
     <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.39370078740157499" right="0.39370078740157499" top="0.39370078740157499" bottom="0.39370078740157499" header="0.39370078740157499" footer="0.39370078740157499"/>
-  <pageSetup paperSize="9" scale="58" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="59" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
Rewizja zestawu krajowego - Cel 14 (pliki Excel, PDF)
</commit_message>
<xml_diff>
--- a/assets/excel/en/national_sdg_indicators.xlsx
+++ b/assets/excel/en/national_sdg_indicators.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sidwab\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C68FBFFF-6B7A-4C44-A574-432027A15113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A037913B-D2A7-433F-86BC-9F6E5E42A691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2104" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2153" uniqueCount="441">
   <si>
     <t>sdg.gov.pl/en</t>
   </si>
@@ -1108,10 +1108,25 @@
     <t>proportion of stocks overexploited on the Baltic Sea</t>
   </si>
   <si>
+    <t>14.1.b Share of marine protected areas</t>
+  </si>
+  <si>
     <t>Increase of maritime economy share in GDP and increase of employment in maritime economy</t>
   </si>
   <si>
-    <t>14.2.a Indices of average employment in maritime economy (2010=100)</t>
+    <t>14.2.a Indices of average employment in the maritime economy (previous year = 100)</t>
+  </si>
+  <si>
+    <t>private</t>
+  </si>
+  <si>
+    <t>previous year = 100</t>
+  </si>
+  <si>
+    <t>public</t>
+  </si>
+  <si>
+    <t>14.2.b Share of the maritime economy in the gross value of fixed assets of the national economy</t>
   </si>
   <si>
     <t>Enhancement of Polish seaports position, increase in competitiveness of sea transport and ensurance of sea security</t>
@@ -1123,6 +1138,21 @@
     <t xml:space="preserve">million tonnes [mln t] </t>
   </si>
   <si>
+    <t>14.3.b Domestic passenger traffic in seaports</t>
+  </si>
+  <si>
+    <t>by passenger traffic</t>
+  </si>
+  <si>
+    <t>arrivals</t>
+  </si>
+  <si>
+    <t>departures</t>
+  </si>
+  <si>
+    <t>14.3.c International passenger traffic in seaports</t>
+  </si>
+  <si>
     <t>Goal 15. Life on land</t>
   </si>
   <si>
@@ -1321,7 +1351,7 @@
     <t>The Ministry of Economic Development and Technology / The Chancellery of the  Prime Minister</t>
   </si>
   <si>
-    <t>Last update: 05-08-2026, 13:23</t>
+    <t>Last update: 07-08-2026, 10:19</t>
   </si>
 </sst>
 </file>
@@ -1867,7 +1897,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W302"/>
+  <dimension ref="A1:W309"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" customWidth="1"/>
@@ -18330,15 +18360,15 @@
         <v>355</v>
       </c>
     </row>
-    <row r="264" spans="1:23" ht="18" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:23" ht="72" x14ac:dyDescent="0.25">
       <c r="A264" s="2" t="s">
         <v>350</v>
       </c>
       <c r="B264" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="C264" s="2" t="s">
         <v>359</v>
-      </c>
-      <c r="C264" s="2" t="s">
-        <v>360</v>
       </c>
       <c r="D264" s="2" t="s">
         <v>27</v>
@@ -18347,205 +18377,183 @@
         <v>28</v>
       </c>
       <c r="F264" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="G264" s="4">
-        <v>100</v>
-      </c>
-      <c r="H264" s="4">
-        <v>100.8</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="G264" s="3"/>
+      <c r="H264" s="3"/>
       <c r="I264" s="4">
-        <v>99.9</v>
-      </c>
-      <c r="J264" s="4">
-        <v>101.8</v>
-      </c>
-      <c r="K264" s="4">
-        <v>104.9</v>
-      </c>
-      <c r="L264" s="4">
-        <v>106</v>
-      </c>
+        <v>21.8</v>
+      </c>
+      <c r="J264" s="3"/>
+      <c r="K264" s="3"/>
+      <c r="L264" s="3"/>
       <c r="M264" s="4">
-        <v>119.9</v>
-      </c>
-      <c r="N264" s="4">
-        <v>119.4</v>
-      </c>
-      <c r="O264" s="4">
-        <v>130</v>
-      </c>
+        <v>21.8</v>
+      </c>
+      <c r="N264" s="3"/>
+      <c r="O264" s="3"/>
       <c r="P264" s="4">
-        <v>189.5</v>
-      </c>
-      <c r="Q264" s="4">
-        <v>186.6</v>
-      </c>
+        <v>21.8</v>
+      </c>
+      <c r="Q264" s="3"/>
       <c r="R264" s="4">
-        <v>190.1</v>
+        <v>21.9</v>
       </c>
       <c r="S264" s="4">
-        <v>200.8</v>
+        <v>21.9</v>
       </c>
       <c r="T264" s="4">
-        <v>205.6</v>
-      </c>
-      <c r="U264" s="4">
-        <v>208.5</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="U264" s="3"/>
       <c r="V264" s="3"/>
       <c r="W264" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="265" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="265" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A265" s="2" t="s">
         <v>350</v>
       </c>
       <c r="B265" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="C265" s="2" t="s">
         <v>361</v>
       </c>
-      <c r="C265" s="2" t="s">
+      <c r="D265" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="E265" s="3" t="s">
         <v>362</v>
-      </c>
-      <c r="D265" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E265" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="F265" s="3" t="s">
         <v>363</v>
       </c>
-      <c r="G265" s="4">
-        <v>59.5</v>
-      </c>
+      <c r="G265" s="3"/>
       <c r="H265" s="4">
-        <v>57.7</v>
+        <v>101.8</v>
       </c>
       <c r="I265" s="4">
-        <v>58.8</v>
+        <v>100</v>
       </c>
       <c r="J265" s="4">
-        <v>64.3</v>
+        <v>101.8</v>
       </c>
       <c r="K265" s="4">
-        <v>68.7</v>
+        <v>103.2</v>
       </c>
       <c r="L265" s="4">
-        <v>69.5</v>
+        <v>101.8</v>
       </c>
       <c r="M265" s="4">
-        <v>72.900000000000006</v>
+        <v>115.4</v>
       </c>
       <c r="N265" s="4">
-        <v>78.099999999999994</v>
+        <v>98.6</v>
       </c>
       <c r="O265" s="4">
-        <v>91.8</v>
+        <v>110.3</v>
       </c>
       <c r="P265" s="4">
-        <v>93.9</v>
+        <v>149.6</v>
       </c>
       <c r="Q265" s="4">
-        <v>88.5</v>
+        <v>98.5</v>
       </c>
       <c r="R265" s="4">
-        <v>96.7</v>
+        <v>102.3</v>
       </c>
       <c r="S265" s="4">
-        <v>119</v>
+        <v>106.1</v>
       </c>
       <c r="T265" s="4">
-        <v>136.4</v>
+        <v>102.7</v>
       </c>
       <c r="U265" s="4">
-        <v>124.2</v>
+        <v>101</v>
       </c>
       <c r="V265" s="3"/>
       <c r="W265" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="266" spans="1:23" ht="36" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A266" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="B266" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="C266" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D266" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="E266" s="3" t="s">
         <v>364</v>
       </c>
-      <c r="B266" s="2" t="s">
-        <v>365</v>
-      </c>
-      <c r="C266" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="D266" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E266" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="F266" s="3" t="s">
-        <v>367</v>
-      </c>
-      <c r="G266" s="4">
-        <v>90.8</v>
-      </c>
+        <v>363</v>
+      </c>
+      <c r="G266" s="3"/>
       <c r="H266" s="4">
-        <v>88.8</v>
+        <v>95.6</v>
       </c>
       <c r="I266" s="4">
-        <v>86.5</v>
+        <v>94.8</v>
       </c>
       <c r="J266" s="4">
-        <v>87</v>
+        <v>102.6</v>
       </c>
       <c r="K266" s="4">
-        <v>85</v>
+        <v>102.1</v>
       </c>
       <c r="L266" s="4">
-        <v>87.4</v>
+        <v>96.9</v>
       </c>
       <c r="M266" s="4">
-        <v>88.7</v>
+        <v>99.7</v>
       </c>
       <c r="N266" s="4">
-        <v>84.6</v>
+        <v>106.1</v>
       </c>
       <c r="O266" s="4">
-        <v>77.3</v>
+        <v>100.5</v>
       </c>
       <c r="P266" s="4">
-        <v>79.7</v>
+        <v>119</v>
       </c>
       <c r="Q266" s="4">
-        <v>81.900000000000006</v>
+        <v>98.4</v>
       </c>
       <c r="R266" s="4">
-        <v>74.8</v>
+        <v>98.1</v>
       </c>
       <c r="S266" s="4">
-        <v>77</v>
+        <v>101.5</v>
       </c>
       <c r="T266" s="4">
-        <v>77.2</v>
+        <v>98.9</v>
       </c>
       <c r="U266" s="4">
-        <v>76.3</v>
+        <v>105.5</v>
       </c>
       <c r="V266" s="3"/>
       <c r="W266" s="2" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="267" spans="1:23" ht="36" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="267" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A267" s="2" t="s">
-        <v>364</v>
+        <v>350</v>
       </c>
       <c r="B267" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="C267" s="2" t="s">
         <v>365</v>
-      </c>
-      <c r="C267" s="2" t="s">
-        <v>369</v>
       </c>
       <c r="D267" s="2" t="s">
         <v>27</v>
@@ -18556,65 +18564,65 @@
       <c r="F267" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G267" s="7">
-        <v>0.19600000000000001</v>
-      </c>
-      <c r="H267" s="7">
-        <v>0.20499999999999999</v>
-      </c>
-      <c r="I267" s="7">
-        <v>0.20599999999999999</v>
-      </c>
-      <c r="J267" s="7">
-        <v>0.19800000000000001</v>
-      </c>
-      <c r="K267" s="7">
-        <v>0.20100000000000001</v>
-      </c>
-      <c r="L267" s="7">
-        <v>0.20300000000000001</v>
-      </c>
-      <c r="M267" s="7">
-        <v>0.20699999999999999</v>
-      </c>
-      <c r="N267" s="7">
-        <v>0.19800000000000001</v>
-      </c>
-      <c r="O267" s="7">
-        <v>0.19800000000000001</v>
-      </c>
-      <c r="P267" s="7">
-        <v>0.19900000000000001</v>
-      </c>
-      <c r="Q267" s="7">
-        <v>0.2</v>
-      </c>
-      <c r="R267" s="7">
-        <v>0.19900000000000001</v>
-      </c>
-      <c r="S267" s="7">
-        <v>0.19800000000000001</v>
-      </c>
-      <c r="T267" s="7">
-        <v>0.192</v>
-      </c>
-      <c r="U267" s="7">
-        <v>0.192</v>
+      <c r="G267" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="H267" s="4">
+        <v>0.6</v>
+      </c>
+      <c r="I267" s="4">
+        <v>0.6</v>
+      </c>
+      <c r="J267" s="4">
+        <v>0.6</v>
+      </c>
+      <c r="K267" s="4">
+        <v>0.6</v>
+      </c>
+      <c r="L267" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="M267" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="N267" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="O267" s="4">
+        <v>0.8</v>
+      </c>
+      <c r="P267" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="Q267" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="R267" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="S267" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="T267" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="U267" s="4">
+        <v>0.8</v>
       </c>
       <c r="V267" s="3"/>
       <c r="W267" s="2" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="268" spans="1:23" ht="36" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="268" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A268" s="2" t="s">
-        <v>364</v>
+        <v>350</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="D268" s="2" t="s">
         <v>27</v>
@@ -18623,343 +18631,351 @@
         <v>28</v>
       </c>
       <c r="F268" s="3" t="s">
-        <v>34</v>
+        <v>368</v>
       </c>
       <c r="G268" s="4">
-        <v>30.5</v>
+        <v>59.5</v>
       </c>
       <c r="H268" s="4">
-        <v>30.5</v>
+        <v>57.7</v>
       </c>
       <c r="I268" s="4">
-        <v>30.6</v>
+        <v>58.8</v>
       </c>
       <c r="J268" s="4">
-        <v>30.6</v>
+        <v>64.3</v>
       </c>
       <c r="K268" s="4">
-        <v>30.7</v>
+        <v>68.7</v>
       </c>
       <c r="L268" s="4">
-        <v>30.8</v>
+        <v>69.5</v>
       </c>
       <c r="M268" s="4">
-        <v>30.8</v>
+        <v>72.900000000000006</v>
       </c>
       <c r="N268" s="4">
-        <v>30.9</v>
+        <v>78.099999999999994</v>
       </c>
       <c r="O268" s="4">
-        <v>30.9</v>
+        <v>91.8</v>
       </c>
       <c r="P268" s="4">
-        <v>30.9</v>
+        <v>93.9</v>
       </c>
       <c r="Q268" s="4">
-        <v>30.9</v>
+        <v>88.5</v>
       </c>
       <c r="R268" s="4">
-        <v>30.9</v>
+        <v>96.7</v>
       </c>
       <c r="S268" s="4">
-        <v>31</v>
+        <v>119</v>
       </c>
       <c r="T268" s="4">
-        <v>31</v>
+        <v>136.4</v>
       </c>
       <c r="U268" s="4">
-        <v>31</v>
+        <v>124.2</v>
       </c>
       <c r="V268" s="3"/>
       <c r="W268" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="269" spans="1:23" ht="36" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A269" s="2" t="s">
-        <v>364</v>
+        <v>350</v>
       </c>
       <c r="B269" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="C269" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="D269" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="E269" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="F269" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G269" s="6">
+        <v>493249</v>
+      </c>
+      <c r="H269" s="6">
+        <v>474154</v>
+      </c>
+      <c r="I269" s="6">
+        <v>372834</v>
+      </c>
+      <c r="J269" s="6">
+        <v>302421</v>
+      </c>
+      <c r="K269" s="6">
+        <v>232736</v>
+      </c>
+      <c r="L269" s="6">
+        <v>284915</v>
+      </c>
+      <c r="M269" s="6">
+        <v>334020</v>
+      </c>
+      <c r="N269" s="6">
+        <v>279852</v>
+      </c>
+      <c r="O269" s="6">
+        <v>330941</v>
+      </c>
+      <c r="P269" s="6">
+        <v>351775</v>
+      </c>
+      <c r="Q269" s="6">
+        <v>176029</v>
+      </c>
+      <c r="R269" s="6">
+        <v>275628</v>
+      </c>
+      <c r="S269" s="6">
+        <v>257955</v>
+      </c>
+      <c r="T269" s="6">
+        <v>261424</v>
+      </c>
+      <c r="U269" s="6">
+        <v>353616</v>
+      </c>
+      <c r="V269" s="6">
+        <v>303091</v>
+      </c>
+      <c r="W269" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="270" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+      <c r="A270" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="B270" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="C270" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="D270" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="E270" s="3" t="s">
         <v>372</v>
       </c>
-      <c r="C269" s="2" t="s">
-        <v>373</v>
-      </c>
-      <c r="D269" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E269" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F269" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="G269" s="6">
-        <v>28</v>
-      </c>
-      <c r="H269" s="6">
-        <v>27</v>
-      </c>
-      <c r="I269" s="6">
-        <v>26</v>
-      </c>
-      <c r="J269" s="6">
-        <v>25</v>
-      </c>
-      <c r="K269" s="6">
-        <v>24</v>
-      </c>
-      <c r="L269" s="6">
-        <v>23</v>
-      </c>
-      <c r="M269" s="6">
-        <v>22</v>
-      </c>
-      <c r="N269" s="6">
-        <v>22</v>
-      </c>
-      <c r="O269" s="6">
-        <v>22</v>
-      </c>
-      <c r="P269" s="6">
-        <v>21</v>
-      </c>
-      <c r="Q269" s="6">
-        <v>19</v>
-      </c>
-      <c r="R269" s="6">
-        <v>17</v>
-      </c>
-      <c r="S269" s="6">
-        <v>16</v>
-      </c>
-      <c r="T269" s="6">
-        <v>16</v>
-      </c>
-      <c r="U269" s="6">
-        <v>15</v>
-      </c>
-      <c r="V269" s="3"/>
-      <c r="W269" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="270" spans="1:23" ht="36" x14ac:dyDescent="0.25">
-      <c r="A270" s="2" t="s">
-        <v>364</v>
-      </c>
-      <c r="B270" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="C270" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="D270" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E270" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="F270" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G270" s="4">
-        <v>64.7</v>
-      </c>
-      <c r="H270" s="4">
-        <v>65.7</v>
-      </c>
-      <c r="I270" s="4">
-        <v>68.599999999999994</v>
-      </c>
-      <c r="J270" s="4">
-        <v>70.3</v>
-      </c>
-      <c r="K270" s="4">
-        <v>71.5</v>
-      </c>
-      <c r="L270" s="4">
-        <v>72.7</v>
-      </c>
-      <c r="M270" s="4">
-        <v>73.5</v>
-      </c>
-      <c r="N270" s="4">
-        <v>73.599999999999994</v>
-      </c>
-      <c r="O270" s="4">
-        <v>74</v>
-      </c>
-      <c r="P270" s="4">
-        <v>74.5</v>
-      </c>
-      <c r="Q270" s="4">
-        <v>74.900000000000006</v>
-      </c>
-      <c r="R270" s="4">
-        <v>75.2</v>
-      </c>
-      <c r="S270" s="4">
-        <v>75.7</v>
-      </c>
-      <c r="T270" s="4">
-        <v>75.900000000000006</v>
-      </c>
-      <c r="U270" s="4">
-        <v>76.2</v>
-      </c>
-      <c r="V270" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="G270" s="6">
+        <v>485152</v>
+      </c>
+      <c r="H270" s="6">
+        <v>474731</v>
+      </c>
+      <c r="I270" s="6">
+        <v>372768</v>
+      </c>
+      <c r="J270" s="6">
+        <v>301883</v>
+      </c>
+      <c r="K270" s="6">
+        <v>233889</v>
+      </c>
+      <c r="L270" s="6">
+        <v>285054</v>
+      </c>
+      <c r="M270" s="6">
+        <v>334120</v>
+      </c>
+      <c r="N270" s="6">
+        <v>279520</v>
+      </c>
+      <c r="O270" s="6">
+        <v>330602</v>
+      </c>
+      <c r="P270" s="6">
+        <v>351685</v>
+      </c>
+      <c r="Q270" s="6">
+        <v>175421</v>
+      </c>
+      <c r="R270" s="6">
+        <v>276413</v>
+      </c>
+      <c r="S270" s="6">
+        <v>262425</v>
+      </c>
+      <c r="T270" s="6">
+        <v>256157</v>
+      </c>
+      <c r="U270" s="6">
+        <v>346671</v>
+      </c>
+      <c r="V270" s="6">
+        <v>299556</v>
+      </c>
       <c r="W270" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="271" spans="1:23" ht="36" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A271" s="2" t="s">
-        <v>364</v>
+        <v>350</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>372</v>
+        <v>366</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D271" s="2" t="s">
-        <v>37</v>
+        <v>370</v>
       </c>
       <c r="E271" s="3" t="s">
-        <v>39</v>
+        <v>371</v>
       </c>
       <c r="F271" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G271" s="4">
-        <v>88</v>
-      </c>
-      <c r="H271" s="4">
-        <v>88.4</v>
-      </c>
-      <c r="I271" s="4">
-        <v>91.7</v>
-      </c>
-      <c r="J271" s="4">
-        <v>93.3</v>
-      </c>
-      <c r="K271" s="4">
-        <v>93.9</v>
-      </c>
-      <c r="L271" s="4">
-        <v>94.6</v>
-      </c>
-      <c r="M271" s="4">
-        <v>94.8</v>
-      </c>
-      <c r="N271" s="4">
-        <v>94.5</v>
-      </c>
-      <c r="O271" s="4">
-        <v>94.6</v>
-      </c>
-      <c r="P271" s="4">
-        <v>94.8</v>
-      </c>
-      <c r="Q271" s="4">
-        <v>94.7</v>
-      </c>
-      <c r="R271" s="4">
-        <v>94.6</v>
-      </c>
-      <c r="S271" s="4">
-        <v>95</v>
-      </c>
-      <c r="T271" s="4">
-        <v>94.8</v>
-      </c>
-      <c r="U271" s="4">
-        <v>94.6</v>
-      </c>
-      <c r="V271" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="G271" s="6">
+        <v>759502</v>
+      </c>
+      <c r="H271" s="6">
+        <v>781353</v>
+      </c>
+      <c r="I271" s="6">
+        <v>802702</v>
+      </c>
+      <c r="J271" s="6">
+        <v>787070</v>
+      </c>
+      <c r="K271" s="6">
+        <v>875518</v>
+      </c>
+      <c r="L271" s="6">
+        <v>919666</v>
+      </c>
+      <c r="M271" s="6">
+        <v>962501</v>
+      </c>
+      <c r="N271" s="6">
+        <v>1011758</v>
+      </c>
+      <c r="O271" s="6">
+        <v>1029218</v>
+      </c>
+      <c r="P271" s="6">
+        <v>1057440</v>
+      </c>
+      <c r="Q271" s="6">
+        <v>780543</v>
+      </c>
+      <c r="R271" s="6">
+        <v>882463</v>
+      </c>
+      <c r="S271" s="6">
+        <v>885794</v>
+      </c>
+      <c r="T271" s="6">
+        <v>871811</v>
+      </c>
+      <c r="U271" s="6">
+        <v>872944</v>
+      </c>
+      <c r="V271" s="6">
+        <v>884918</v>
+      </c>
       <c r="W271" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="272" spans="1:23" ht="36" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A272" s="2" t="s">
-        <v>364</v>
+        <v>350</v>
       </c>
       <c r="B272" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="C272" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="D272" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="E272" s="3" t="s">
         <v>372</v>
       </c>
-      <c r="C272" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="D272" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E272" s="3" t="s">
-        <v>40</v>
-      </c>
       <c r="F272" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G272" s="4">
-        <v>28.5</v>
-      </c>
-      <c r="H272" s="4">
-        <v>30.6</v>
-      </c>
-      <c r="I272" s="4">
-        <v>33.1</v>
-      </c>
-      <c r="J272" s="4">
-        <v>35.299999999999997</v>
-      </c>
-      <c r="K272" s="4">
-        <v>37.4</v>
-      </c>
-      <c r="L272" s="4">
-        <v>39.6</v>
-      </c>
-      <c r="M272" s="4">
-        <v>41.2</v>
-      </c>
-      <c r="N272" s="4">
-        <v>42</v>
-      </c>
-      <c r="O272" s="4">
-        <v>42.9</v>
-      </c>
-      <c r="P272" s="4">
-        <v>44</v>
-      </c>
-      <c r="Q272" s="4">
-        <v>45.4</v>
-      </c>
-      <c r="R272" s="4">
-        <v>46.5</v>
-      </c>
-      <c r="S272" s="4">
-        <v>47.2</v>
-      </c>
-      <c r="T272" s="4">
-        <v>48.2</v>
-      </c>
-      <c r="U272" s="4">
-        <v>49.3</v>
-      </c>
-      <c r="V272" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="G272" s="6">
+        <v>781553</v>
+      </c>
+      <c r="H272" s="6">
+        <v>802785</v>
+      </c>
+      <c r="I272" s="6">
+        <v>809836</v>
+      </c>
+      <c r="J272" s="6">
+        <v>809712</v>
+      </c>
+      <c r="K272" s="6">
+        <v>878045</v>
+      </c>
+      <c r="L272" s="6">
+        <v>931632</v>
+      </c>
+      <c r="M272" s="6">
+        <v>970959</v>
+      </c>
+      <c r="N272" s="6">
+        <v>1013639</v>
+      </c>
+      <c r="O272" s="6">
+        <v>1029660</v>
+      </c>
+      <c r="P272" s="6">
+        <v>1026283</v>
+      </c>
+      <c r="Q272" s="6">
+        <v>773182</v>
+      </c>
+      <c r="R272" s="6">
+        <v>881969</v>
+      </c>
+      <c r="S272" s="6">
+        <v>929215</v>
+      </c>
+      <c r="T272" s="6">
+        <v>862113</v>
+      </c>
+      <c r="U272" s="6">
+        <v>853481</v>
+      </c>
+      <c r="V272" s="6">
+        <v>873943</v>
+      </c>
       <c r="W272" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="273" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A273" s="2" t="s">
-        <v>364</v>
+        <v>374</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D273" s="2" t="s">
         <v>27</v>
@@ -18968,67 +18984,67 @@
         <v>28</v>
       </c>
       <c r="F273" s="3" t="s">
-        <v>34</v>
+        <v>377</v>
       </c>
       <c r="G273" s="4">
-        <v>65.7</v>
+        <v>90.8</v>
       </c>
       <c r="H273" s="4">
-        <v>64.8</v>
+        <v>88.8</v>
       </c>
       <c r="I273" s="4">
-        <v>67.400000000000006</v>
+        <v>86.5</v>
       </c>
       <c r="J273" s="4">
-        <v>69.8</v>
+        <v>87</v>
       </c>
       <c r="K273" s="4">
-        <v>70.5</v>
+        <v>85</v>
       </c>
       <c r="L273" s="4">
-        <v>70.900000000000006</v>
+        <v>87.4</v>
       </c>
       <c r="M273" s="4">
-        <v>71.400000000000006</v>
+        <v>88.7</v>
       </c>
       <c r="N273" s="4">
-        <v>72.5</v>
+        <v>84.6</v>
       </c>
       <c r="O273" s="4">
-        <v>73.2</v>
+        <v>77.3</v>
       </c>
       <c r="P273" s="4">
-        <v>73.900000000000006</v>
+        <v>79.7</v>
       </c>
       <c r="Q273" s="4">
-        <v>73.3</v>
+        <v>81.900000000000006</v>
       </c>
       <c r="R273" s="4">
-        <v>72.8</v>
+        <v>74.8</v>
       </c>
       <c r="S273" s="4">
+        <v>77</v>
+      </c>
+      <c r="T273" s="4">
+        <v>77.2</v>
+      </c>
+      <c r="U273" s="4">
         <v>76.3</v>
-      </c>
-      <c r="T273" s="4">
-        <v>78.099999999999994</v>
-      </c>
-      <c r="U273" s="4">
-        <v>78.599999999999994</v>
       </c>
       <c r="V273" s="3"/>
       <c r="W273" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="274" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="274" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A274" s="2" t="s">
-        <v>364</v>
+        <v>374</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D274" s="2" t="s">
         <v>27</v>
@@ -19037,67 +19053,67 @@
         <v>28</v>
       </c>
       <c r="F274" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="G274" s="6">
-        <v>70108</v>
-      </c>
-      <c r="H274" s="6">
-        <v>248240</v>
-      </c>
-      <c r="I274" s="6">
-        <v>168221</v>
-      </c>
-      <c r="J274" s="6">
-        <v>72837</v>
-      </c>
-      <c r="K274" s="6">
-        <v>64283</v>
-      </c>
-      <c r="L274" s="6">
-        <v>68694</v>
-      </c>
-      <c r="M274" s="6">
-        <v>60135</v>
-      </c>
-      <c r="N274" s="6">
-        <v>46337</v>
-      </c>
-      <c r="O274" s="6">
-        <v>50289</v>
-      </c>
-      <c r="P274" s="6">
-        <v>104107</v>
-      </c>
-      <c r="Q274" s="6">
-        <v>201963</v>
-      </c>
-      <c r="R274" s="6">
-        <v>84506</v>
-      </c>
-      <c r="S274" s="6">
-        <v>295948</v>
-      </c>
-      <c r="T274" s="6">
-        <v>123796</v>
-      </c>
-      <c r="U274" s="6">
-        <v>104040</v>
+        <v>34</v>
+      </c>
+      <c r="G274" s="7">
+        <v>0.19600000000000001</v>
+      </c>
+      <c r="H274" s="7">
+        <v>0.20499999999999999</v>
+      </c>
+      <c r="I274" s="7">
+        <v>0.20599999999999999</v>
+      </c>
+      <c r="J274" s="7">
+        <v>0.19800000000000001</v>
+      </c>
+      <c r="K274" s="7">
+        <v>0.20100000000000001</v>
+      </c>
+      <c r="L274" s="7">
+        <v>0.20300000000000001</v>
+      </c>
+      <c r="M274" s="7">
+        <v>0.20699999999999999</v>
+      </c>
+      <c r="N274" s="7">
+        <v>0.19800000000000001</v>
+      </c>
+      <c r="O274" s="7">
+        <v>0.19800000000000001</v>
+      </c>
+      <c r="P274" s="7">
+        <v>0.19900000000000001</v>
+      </c>
+      <c r="Q274" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="R274" s="7">
+        <v>0.19900000000000001</v>
+      </c>
+      <c r="S274" s="7">
+        <v>0.19800000000000001</v>
+      </c>
+      <c r="T274" s="7">
+        <v>0.192</v>
+      </c>
+      <c r="U274" s="7">
+        <v>0.192</v>
       </c>
       <c r="V274" s="3"/>
       <c r="W274" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="275" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="275" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A275" s="2" t="s">
-        <v>364</v>
+        <v>374</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="D275" s="2" t="s">
         <v>27</v>
@@ -19109,64 +19125,64 @@
         <v>34</v>
       </c>
       <c r="G275" s="4">
-        <v>2.9</v>
+        <v>30.5</v>
       </c>
       <c r="H275" s="4">
-        <v>3.8</v>
+        <v>30.5</v>
       </c>
       <c r="I275" s="4">
-        <v>6</v>
+        <v>30.6</v>
       </c>
       <c r="J275" s="4">
-        <v>4.3</v>
+        <v>30.6</v>
       </c>
       <c r="K275" s="4">
-        <v>4.5999999999999996</v>
+        <v>30.7</v>
       </c>
       <c r="L275" s="4">
-        <v>4.2</v>
+        <v>30.8</v>
       </c>
       <c r="M275" s="4">
-        <v>3.1</v>
+        <v>30.8</v>
       </c>
       <c r="N275" s="4">
-        <v>3</v>
+        <v>30.9</v>
       </c>
       <c r="O275" s="4">
-        <v>3.2</v>
+        <v>30.9</v>
       </c>
       <c r="P275" s="4">
-        <v>3.4</v>
+        <v>30.9</v>
       </c>
       <c r="Q275" s="4">
-        <v>3.2</v>
+        <v>30.9</v>
       </c>
       <c r="R275" s="4">
-        <v>4.5</v>
+        <v>30.9</v>
       </c>
       <c r="S275" s="4">
-        <v>6.6</v>
+        <v>31</v>
       </c>
       <c r="T275" s="4">
-        <v>5.8</v>
+        <v>31</v>
       </c>
       <c r="U275" s="4">
-        <v>4.5</v>
+        <v>31</v>
       </c>
       <c r="V275" s="3"/>
       <c r="W275" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="276" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A276" s="2" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D276" s="2" t="s">
         <v>27</v>
@@ -19175,72 +19191,70 @@
         <v>28</v>
       </c>
       <c r="F276" s="3" t="s">
-        <v>34</v>
+        <v>106</v>
       </c>
       <c r="G276" s="6">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="H276" s="6">
-        <v>75</v>
+        <v>27</v>
       </c>
       <c r="I276" s="6">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="J276" s="6">
-        <v>64</v>
+        <v>25</v>
       </c>
       <c r="K276" s="6">
-        <v>70</v>
+        <v>24</v>
       </c>
       <c r="L276" s="6">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="M276" s="6">
-        <v>80</v>
+        <v>22</v>
       </c>
       <c r="N276" s="6">
-        <v>89</v>
+        <v>22</v>
       </c>
       <c r="O276" s="6">
-        <v>86</v>
+        <v>22</v>
       </c>
       <c r="P276" s="6">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="Q276" s="6">
-        <v>85</v>
+        <v>19</v>
       </c>
       <c r="R276" s="6">
-        <v>82</v>
+        <v>17</v>
       </c>
       <c r="S276" s="6">
-        <v>83</v>
+        <v>16</v>
       </c>
       <c r="T276" s="6">
-        <v>88</v>
+        <v>16</v>
       </c>
       <c r="U276" s="6">
-        <v>88</v>
-      </c>
-      <c r="V276" s="6">
-        <v>86</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="V276" s="3"/>
       <c r="W276" s="2" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="277" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="277" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A277" s="2" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C277" s="2" t="s">
         <v>384</v>
       </c>
       <c r="D277" s="2" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E277" s="3" t="s">
         <v>28</v>
@@ -19248,163 +19262,203 @@
       <c r="F277" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G277" s="6">
-        <v>55</v>
-      </c>
-      <c r="H277" s="3"/>
-      <c r="I277" s="6">
-        <v>58</v>
-      </c>
-      <c r="J277" s="3"/>
-      <c r="K277" s="6">
-        <v>60</v>
-      </c>
-      <c r="L277" s="3"/>
-      <c r="M277" s="6">
-        <v>64</v>
-      </c>
-      <c r="N277" s="3"/>
-      <c r="O277" s="6">
-        <v>65</v>
-      </c>
-      <c r="P277" s="3"/>
-      <c r="Q277" s="6">
+      <c r="G277" s="4">
+        <v>64.7</v>
+      </c>
+      <c r="H277" s="4">
+        <v>65.7</v>
+      </c>
+      <c r="I277" s="4">
+        <v>68.599999999999994</v>
+      </c>
+      <c r="J277" s="4">
+        <v>70.3</v>
+      </c>
+      <c r="K277" s="4">
+        <v>71.5</v>
+      </c>
+      <c r="L277" s="4">
+        <v>72.7</v>
+      </c>
+      <c r="M277" s="4">
+        <v>73.5</v>
+      </c>
+      <c r="N277" s="4">
+        <v>73.599999999999994</v>
+      </c>
+      <c r="O277" s="4">
         <v>74</v>
       </c>
-      <c r="R277" s="3"/>
-      <c r="S277" s="6">
-        <v>63</v>
-      </c>
-      <c r="T277" s="3"/>
-      <c r="U277" s="6">
-        <v>71</v>
+      <c r="P277" s="4">
+        <v>74.5</v>
+      </c>
+      <c r="Q277" s="4">
+        <v>74.900000000000006</v>
+      </c>
+      <c r="R277" s="4">
+        <v>75.2</v>
+      </c>
+      <c r="S277" s="4">
+        <v>75.7</v>
+      </c>
+      <c r="T277" s="4">
+        <v>75.900000000000006</v>
+      </c>
+      <c r="U277" s="4">
+        <v>76.2</v>
       </c>
       <c r="V277" s="3"/>
       <c r="W277" s="2" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="278" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="278" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A278" s="2" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D278" s="2" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E278" s="3" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="F278" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G278" s="3"/>
-      <c r="H278" s="3"/>
-      <c r="I278" s="3"/>
-      <c r="J278" s="3"/>
-      <c r="K278" s="3"/>
-      <c r="L278" s="3"/>
-      <c r="M278" s="3"/>
-      <c r="N278" s="3"/>
-      <c r="O278" s="3"/>
-      <c r="P278" s="3"/>
-      <c r="Q278" s="3"/>
-      <c r="R278" s="3"/>
-      <c r="S278" s="5">
-        <v>33109.31</v>
-      </c>
-      <c r="T278" s="5">
-        <v>33829.39</v>
-      </c>
-      <c r="U278" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="G278" s="4">
+        <v>88</v>
+      </c>
+      <c r="H278" s="4">
+        <v>88.4</v>
+      </c>
+      <c r="I278" s="4">
+        <v>91.7</v>
+      </c>
+      <c r="J278" s="4">
+        <v>93.3</v>
+      </c>
+      <c r="K278" s="4">
+        <v>93.9</v>
+      </c>
+      <c r="L278" s="4">
+        <v>94.6</v>
+      </c>
+      <c r="M278" s="4">
+        <v>94.8</v>
+      </c>
+      <c r="N278" s="4">
+        <v>94.5</v>
+      </c>
+      <c r="O278" s="4">
+        <v>94.6</v>
+      </c>
+      <c r="P278" s="4">
+        <v>94.8</v>
+      </c>
+      <c r="Q278" s="4">
+        <v>94.7</v>
+      </c>
+      <c r="R278" s="4">
+        <v>94.6</v>
+      </c>
+      <c r="S278" s="4">
+        <v>95</v>
+      </c>
+      <c r="T278" s="4">
+        <v>94.8</v>
+      </c>
+      <c r="U278" s="4">
+        <v>94.6</v>
+      </c>
       <c r="V278" s="3"/>
       <c r="W278" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="279" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="279" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A279" s="2" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D279" s="2" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E279" s="3" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="F279" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="G279" s="5">
-        <v>1.02</v>
-      </c>
-      <c r="H279" s="5">
-        <v>0.96</v>
-      </c>
-      <c r="I279" s="5">
-        <v>1</v>
-      </c>
-      <c r="J279" s="5">
-        <v>1.05</v>
-      </c>
-      <c r="K279" s="5">
-        <v>1.06</v>
-      </c>
-      <c r="L279" s="5">
-        <v>0.95</v>
-      </c>
-      <c r="M279" s="5">
-        <v>0.91</v>
-      </c>
-      <c r="N279" s="5">
-        <v>0.81</v>
-      </c>
-      <c r="O279" s="5">
-        <v>0.87</v>
-      </c>
-      <c r="P279" s="5">
-        <v>1.01</v>
-      </c>
-      <c r="Q279" s="5">
-        <v>0.85</v>
-      </c>
-      <c r="R279" s="5">
-        <v>0.83</v>
-      </c>
-      <c r="S279" s="5">
-        <v>0.72</v>
-      </c>
-      <c r="T279" s="5">
-        <v>0.78</v>
-      </c>
-      <c r="U279" s="5">
-        <v>0.69</v>
+        <v>34</v>
+      </c>
+      <c r="G279" s="4">
+        <v>28.5</v>
+      </c>
+      <c r="H279" s="4">
+        <v>30.6</v>
+      </c>
+      <c r="I279" s="4">
+        <v>33.1</v>
+      </c>
+      <c r="J279" s="4">
+        <v>35.299999999999997</v>
+      </c>
+      <c r="K279" s="4">
+        <v>37.4</v>
+      </c>
+      <c r="L279" s="4">
+        <v>39.6</v>
+      </c>
+      <c r="M279" s="4">
+        <v>41.2</v>
+      </c>
+      <c r="N279" s="4">
+        <v>42</v>
+      </c>
+      <c r="O279" s="4">
+        <v>42.9</v>
+      </c>
+      <c r="P279" s="4">
+        <v>44</v>
+      </c>
+      <c r="Q279" s="4">
+        <v>45.4</v>
+      </c>
+      <c r="R279" s="4">
+        <v>46.5</v>
+      </c>
+      <c r="S279" s="4">
+        <v>47.2</v>
+      </c>
+      <c r="T279" s="4">
+        <v>48.2</v>
+      </c>
+      <c r="U279" s="4">
+        <v>49.3</v>
       </c>
       <c r="V279" s="3"/>
       <c r="W279" s="2" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="280" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="280" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A280" s="2" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="D280" s="2" t="s">
         <v>27</v>
@@ -19415,65 +19469,65 @@
       <c r="F280" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G280" s="5">
-        <v>1.84</v>
-      </c>
-      <c r="H280" s="5">
-        <v>1.79</v>
-      </c>
-      <c r="I280" s="5">
-        <v>1.8</v>
-      </c>
-      <c r="J280" s="5">
-        <v>1.79</v>
-      </c>
-      <c r="K280" s="5">
-        <v>1.86</v>
-      </c>
-      <c r="L280" s="5">
-        <v>2.21</v>
-      </c>
-      <c r="M280" s="5">
-        <v>1.99</v>
-      </c>
-      <c r="N280" s="5">
-        <v>1.88</v>
-      </c>
-      <c r="O280" s="5">
-        <v>2</v>
-      </c>
-      <c r="P280" s="5">
-        <v>1.96</v>
-      </c>
-      <c r="Q280" s="5">
-        <v>2.21</v>
-      </c>
-      <c r="R280" s="5">
-        <v>2.19</v>
-      </c>
-      <c r="S280" s="5">
-        <v>2.21</v>
-      </c>
-      <c r="T280" s="5">
-        <v>3.27</v>
-      </c>
-      <c r="U280" s="5">
-        <v>4.07</v>
+      <c r="G280" s="4">
+        <v>65.7</v>
+      </c>
+      <c r="H280" s="4">
+        <v>64.8</v>
+      </c>
+      <c r="I280" s="4">
+        <v>67.400000000000006</v>
+      </c>
+      <c r="J280" s="4">
+        <v>69.8</v>
+      </c>
+      <c r="K280" s="4">
+        <v>70.5</v>
+      </c>
+      <c r="L280" s="4">
+        <v>70.900000000000006</v>
+      </c>
+      <c r="M280" s="4">
+        <v>71.400000000000006</v>
+      </c>
+      <c r="N280" s="4">
+        <v>72.5</v>
+      </c>
+      <c r="O280" s="4">
+        <v>73.2</v>
+      </c>
+      <c r="P280" s="4">
+        <v>73.900000000000006</v>
+      </c>
+      <c r="Q280" s="4">
+        <v>73.3</v>
+      </c>
+      <c r="R280" s="4">
+        <v>72.8</v>
+      </c>
+      <c r="S280" s="4">
+        <v>76.3</v>
+      </c>
+      <c r="T280" s="4">
+        <v>78.099999999999994</v>
+      </c>
+      <c r="U280" s="4">
+        <v>78.599999999999994</v>
       </c>
       <c r="V280" s="3"/>
       <c r="W280" s="2" t="s">
-        <v>390</v>
+        <v>30</v>
       </c>
     </row>
     <row r="281" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A281" s="2" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="D281" s="2" t="s">
         <v>27</v>
@@ -19482,44 +19536,70 @@
         <v>28</v>
       </c>
       <c r="F281" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G281" s="3"/>
-      <c r="H281" s="3"/>
-      <c r="I281" s="3"/>
-      <c r="J281" s="3"/>
-      <c r="K281" s="3"/>
-      <c r="L281" s="3"/>
-      <c r="M281" s="3"/>
-      <c r="N281" s="3"/>
-      <c r="O281" s="3"/>
-      <c r="P281" s="3"/>
-      <c r="Q281" s="3"/>
-      <c r="R281" s="3"/>
-      <c r="S281" s="3"/>
-      <c r="T281" s="3"/>
-      <c r="U281" s="4">
-        <v>30.2</v>
-      </c>
-      <c r="V281" s="4">
-        <v>51.3</v>
-      </c>
+        <v>388</v>
+      </c>
+      <c r="G281" s="6">
+        <v>70108</v>
+      </c>
+      <c r="H281" s="6">
+        <v>248240</v>
+      </c>
+      <c r="I281" s="6">
+        <v>168221</v>
+      </c>
+      <c r="J281" s="6">
+        <v>72837</v>
+      </c>
+      <c r="K281" s="6">
+        <v>64283</v>
+      </c>
+      <c r="L281" s="6">
+        <v>68694</v>
+      </c>
+      <c r="M281" s="6">
+        <v>60135</v>
+      </c>
+      <c r="N281" s="6">
+        <v>46337</v>
+      </c>
+      <c r="O281" s="6">
+        <v>50289</v>
+      </c>
+      <c r="P281" s="6">
+        <v>104107</v>
+      </c>
+      <c r="Q281" s="6">
+        <v>201963</v>
+      </c>
+      <c r="R281" s="6">
+        <v>84506</v>
+      </c>
+      <c r="S281" s="6">
+        <v>295948</v>
+      </c>
+      <c r="T281" s="6">
+        <v>123796</v>
+      </c>
+      <c r="U281" s="6">
+        <v>104040</v>
+      </c>
+      <c r="V281" s="3"/>
       <c r="W281" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="282" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A282" s="2" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="D282" s="2" t="s">
-        <v>90</v>
+        <v>27</v>
       </c>
       <c r="E282" s="3" t="s">
         <v>28</v>
@@ -19528,478 +19608,400 @@
         <v>34</v>
       </c>
       <c r="G282" s="4">
-        <v>28.1</v>
+        <v>2.9</v>
       </c>
       <c r="H282" s="4">
-        <v>27.6</v>
+        <v>3.8</v>
       </c>
       <c r="I282" s="4">
-        <v>31.6</v>
+        <v>6</v>
       </c>
       <c r="J282" s="4">
-        <v>22.6</v>
+        <v>4.3</v>
       </c>
       <c r="K282" s="4">
-        <v>26.9</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="L282" s="4">
-        <v>26.6</v>
+        <v>4.2</v>
       </c>
       <c r="M282" s="4">
-        <v>30.2</v>
+        <v>3.1</v>
       </c>
       <c r="N282" s="4">
-        <v>30.8</v>
+        <v>3</v>
       </c>
       <c r="O282" s="4">
-        <v>35.5</v>
+        <v>3.2</v>
       </c>
       <c r="P282" s="4">
-        <v>40.4</v>
+        <v>3.4</v>
       </c>
       <c r="Q282" s="4">
-        <v>41.9</v>
+        <v>3.2</v>
       </c>
       <c r="R282" s="4">
-        <v>47.5</v>
+        <v>4.5</v>
       </c>
       <c r="S282" s="4">
-        <v>55.4</v>
+        <v>6.6</v>
       </c>
       <c r="T282" s="4">
-        <v>58.5</v>
+        <v>5.8</v>
       </c>
       <c r="U282" s="4">
-        <v>61</v>
-      </c>
-      <c r="V282" s="4">
-        <v>61.1</v>
-      </c>
+        <v>4.5</v>
+      </c>
+      <c r="V282" s="3"/>
       <c r="W282" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="283" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A283" s="2" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="B283" s="2" t="s">
         <v>391</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D283" s="2" t="s">
-        <v>90</v>
+        <v>27</v>
       </c>
       <c r="E283" s="3" t="s">
-        <v>394</v>
+        <v>28</v>
       </c>
       <c r="F283" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G283" s="4">
-        <v>31.5</v>
-      </c>
-      <c r="H283" s="4">
-        <v>27.9</v>
-      </c>
-      <c r="I283" s="4">
-        <v>36.799999999999997</v>
-      </c>
-      <c r="J283" s="4">
-        <v>20.2</v>
-      </c>
-      <c r="K283" s="4">
-        <v>23.9</v>
-      </c>
-      <c r="L283" s="4">
-        <v>20.8</v>
-      </c>
-      <c r="M283" s="4">
-        <v>20.5</v>
-      </c>
-      <c r="N283" s="4">
-        <v>22.4</v>
-      </c>
-      <c r="O283" s="4">
-        <v>29.5</v>
-      </c>
-      <c r="P283" s="4">
-        <v>29.8</v>
-      </c>
-      <c r="Q283" s="4">
-        <v>30.9</v>
-      </c>
-      <c r="R283" s="4">
-        <v>35.6</v>
-      </c>
-      <c r="S283" s="4">
-        <v>42.1</v>
-      </c>
-      <c r="T283" s="4">
-        <v>44</v>
-      </c>
-      <c r="U283" s="4">
-        <v>47.7</v>
-      </c>
-      <c r="V283" s="4">
-        <v>48.9</v>
+      <c r="G283" s="6">
+        <v>70</v>
+      </c>
+      <c r="H283" s="6">
+        <v>75</v>
+      </c>
+      <c r="I283" s="6">
+        <v>66</v>
+      </c>
+      <c r="J283" s="6">
+        <v>64</v>
+      </c>
+      <c r="K283" s="6">
+        <v>70</v>
+      </c>
+      <c r="L283" s="6">
+        <v>66</v>
+      </c>
+      <c r="M283" s="6">
+        <v>80</v>
+      </c>
+      <c r="N283" s="6">
+        <v>89</v>
+      </c>
+      <c r="O283" s="6">
+        <v>86</v>
+      </c>
+      <c r="P283" s="6">
+        <v>89</v>
+      </c>
+      <c r="Q283" s="6">
+        <v>85</v>
+      </c>
+      <c r="R283" s="6">
+        <v>82</v>
+      </c>
+      <c r="S283" s="6">
+        <v>83</v>
+      </c>
+      <c r="T283" s="6">
+        <v>88</v>
+      </c>
+      <c r="U283" s="6">
+        <v>88</v>
+      </c>
+      <c r="V283" s="6">
+        <v>86</v>
       </c>
       <c r="W283" s="2" t="s">
-        <v>30</v>
+        <v>393</v>
       </c>
     </row>
     <row r="284" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A284" s="2" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="B284" s="2" t="s">
         <v>391</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D284" s="2" t="s">
-        <v>90</v>
+        <v>27</v>
       </c>
       <c r="E284" s="3" t="s">
-        <v>395</v>
+        <v>28</v>
       </c>
       <c r="F284" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G284" s="4">
-        <v>47.6</v>
-      </c>
-      <c r="H284" s="4">
-        <v>46.2</v>
-      </c>
-      <c r="I284" s="4">
-        <v>50.6</v>
-      </c>
-      <c r="J284" s="4">
-        <v>39</v>
-      </c>
-      <c r="K284" s="4">
-        <v>46</v>
-      </c>
-      <c r="L284" s="4">
-        <v>45</v>
-      </c>
-      <c r="M284" s="4">
-        <v>48.1</v>
-      </c>
-      <c r="N284" s="4">
-        <v>48.1</v>
-      </c>
-      <c r="O284" s="4">
-        <v>53</v>
-      </c>
-      <c r="P284" s="4">
-        <v>58.6</v>
-      </c>
-      <c r="Q284" s="4">
-        <v>59.9</v>
-      </c>
-      <c r="R284" s="4">
-        <v>68.3</v>
-      </c>
-      <c r="S284" s="4">
-        <v>75.2</v>
-      </c>
-      <c r="T284" s="4">
-        <v>81</v>
-      </c>
-      <c r="U284" s="4">
-        <v>81.2</v>
-      </c>
-      <c r="V284" s="4">
-        <v>81.8</v>
-      </c>
+      <c r="G284" s="6">
+        <v>55</v>
+      </c>
+      <c r="H284" s="3"/>
+      <c r="I284" s="6">
+        <v>58</v>
+      </c>
+      <c r="J284" s="3"/>
+      <c r="K284" s="6">
+        <v>60</v>
+      </c>
+      <c r="L284" s="3"/>
+      <c r="M284" s="6">
+        <v>64</v>
+      </c>
+      <c r="N284" s="3"/>
+      <c r="O284" s="6">
+        <v>65</v>
+      </c>
+      <c r="P284" s="3"/>
+      <c r="Q284" s="6">
+        <v>74</v>
+      </c>
+      <c r="R284" s="3"/>
+      <c r="S284" s="6">
+        <v>63</v>
+      </c>
+      <c r="T284" s="3"/>
+      <c r="U284" s="6">
+        <v>71</v>
+      </c>
+      <c r="V284" s="3"/>
       <c r="W284" s="2" t="s">
-        <v>30</v>
+        <v>393</v>
       </c>
     </row>
     <row r="285" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A285" s="2" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="B285" s="2" t="s">
         <v>391</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="D285" s="2" t="s">
-        <v>90</v>
+        <v>27</v>
       </c>
       <c r="E285" s="3" t="s">
-        <v>396</v>
+        <v>28</v>
       </c>
       <c r="F285" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G285" s="4">
-        <v>37.6</v>
-      </c>
-      <c r="H285" s="4">
-        <v>36.9</v>
-      </c>
-      <c r="I285" s="4">
-        <v>45.3</v>
-      </c>
-      <c r="J285" s="4">
-        <v>35.200000000000003</v>
-      </c>
-      <c r="K285" s="4">
-        <v>40.1</v>
-      </c>
-      <c r="L285" s="4">
-        <v>38.6</v>
-      </c>
-      <c r="M285" s="4">
-        <v>40.5</v>
-      </c>
-      <c r="N285" s="4">
-        <v>45</v>
-      </c>
-      <c r="O285" s="4">
-        <v>49.6</v>
-      </c>
-      <c r="P285" s="4">
-        <v>57.6</v>
-      </c>
-      <c r="Q285" s="4">
-        <v>59.4</v>
-      </c>
-      <c r="R285" s="4">
-        <v>65.900000000000006</v>
-      </c>
-      <c r="S285" s="4">
-        <v>75.599999999999994</v>
-      </c>
-      <c r="T285" s="4">
-        <v>78.3</v>
-      </c>
-      <c r="U285" s="4">
-        <v>81.099999999999994</v>
-      </c>
-      <c r="V285" s="4">
-        <v>78.3</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="G285" s="3"/>
+      <c r="H285" s="3"/>
+      <c r="I285" s="3"/>
+      <c r="J285" s="3"/>
+      <c r="K285" s="3"/>
+      <c r="L285" s="3"/>
+      <c r="M285" s="3"/>
+      <c r="N285" s="3"/>
+      <c r="O285" s="3"/>
+      <c r="P285" s="3"/>
+      <c r="Q285" s="3"/>
+      <c r="R285" s="3"/>
+      <c r="S285" s="5">
+        <v>33109.31</v>
+      </c>
+      <c r="T285" s="5">
+        <v>33829.39</v>
+      </c>
+      <c r="U285" s="3"/>
+      <c r="V285" s="3"/>
       <c r="W285" s="2" t="s">
-        <v>30</v>
+        <v>87</v>
       </c>
     </row>
     <row r="286" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A286" s="2" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="D286" s="2" t="s">
-        <v>90</v>
+        <v>27</v>
       </c>
       <c r="E286" s="3" t="s">
-        <v>397</v>
+        <v>28</v>
       </c>
       <c r="F286" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G286" s="4">
-        <v>26.2</v>
-      </c>
-      <c r="H286" s="4">
-        <v>26.3</v>
-      </c>
-      <c r="I286" s="4">
-        <v>28.7</v>
-      </c>
-      <c r="J286" s="4">
-        <v>21.5</v>
-      </c>
-      <c r="K286" s="4">
-        <v>26.2</v>
-      </c>
-      <c r="L286" s="4">
-        <v>26</v>
-      </c>
-      <c r="M286" s="4">
-        <v>30</v>
-      </c>
-      <c r="N286" s="4">
-        <v>28</v>
-      </c>
-      <c r="O286" s="4">
-        <v>35</v>
-      </c>
-      <c r="P286" s="4">
-        <v>41.4</v>
-      </c>
-      <c r="Q286" s="4">
-        <v>45.1</v>
-      </c>
-      <c r="R286" s="4">
-        <v>51.7</v>
-      </c>
-      <c r="S286" s="4">
-        <v>62.4</v>
-      </c>
-      <c r="T286" s="4">
-        <v>65.7</v>
-      </c>
-      <c r="U286" s="4">
-        <v>68.8</v>
-      </c>
-      <c r="V286" s="4">
-        <v>69.900000000000006</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="G286" s="5">
+        <v>1.02</v>
+      </c>
+      <c r="H286" s="5">
+        <v>0.96</v>
+      </c>
+      <c r="I286" s="5">
+        <v>1</v>
+      </c>
+      <c r="J286" s="5">
+        <v>1.05</v>
+      </c>
+      <c r="K286" s="5">
+        <v>1.06</v>
+      </c>
+      <c r="L286" s="5">
+        <v>0.95</v>
+      </c>
+      <c r="M286" s="5">
+        <v>0.91</v>
+      </c>
+      <c r="N286" s="5">
+        <v>0.81</v>
+      </c>
+      <c r="O286" s="5">
+        <v>0.87</v>
+      </c>
+      <c r="P286" s="5">
+        <v>1.01</v>
+      </c>
+      <c r="Q286" s="5">
+        <v>0.85</v>
+      </c>
+      <c r="R286" s="5">
+        <v>0.83</v>
+      </c>
+      <c r="S286" s="5">
+        <v>0.72</v>
+      </c>
+      <c r="T286" s="5">
+        <v>0.78</v>
+      </c>
+      <c r="U286" s="5">
+        <v>0.69</v>
+      </c>
+      <c r="V286" s="3"/>
       <c r="W286" s="2" t="s">
-        <v>30</v>
+        <v>206</v>
       </c>
     </row>
     <row r="287" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A287" s="2" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="D287" s="2" t="s">
-        <v>90</v>
+        <v>27</v>
       </c>
       <c r="E287" s="3" t="s">
-        <v>398</v>
+        <v>28</v>
       </c>
       <c r="F287" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G287" s="4">
-        <v>13.5</v>
-      </c>
-      <c r="H287" s="4">
-        <v>15.7</v>
-      </c>
-      <c r="I287" s="4">
-        <v>17.2</v>
-      </c>
-      <c r="J287" s="4">
-        <v>12.7</v>
-      </c>
-      <c r="K287" s="4">
-        <v>15.5</v>
-      </c>
-      <c r="L287" s="4">
-        <v>18.3</v>
-      </c>
-      <c r="M287" s="4">
-        <v>19.8</v>
-      </c>
-      <c r="N287" s="4">
-        <v>18.8</v>
-      </c>
-      <c r="O287" s="4">
-        <v>22.4</v>
-      </c>
-      <c r="P287" s="4">
-        <v>28.5</v>
-      </c>
-      <c r="Q287" s="4">
-        <v>29.4</v>
-      </c>
-      <c r="R287" s="4">
-        <v>35</v>
-      </c>
-      <c r="S287" s="4">
-        <v>39.5</v>
-      </c>
-      <c r="T287" s="4">
-        <v>44.4</v>
-      </c>
-      <c r="U287" s="4">
-        <v>50.8</v>
-      </c>
-      <c r="V287" s="4">
-        <v>51.4</v>
-      </c>
+      <c r="G287" s="5">
+        <v>1.84</v>
+      </c>
+      <c r="H287" s="5">
+        <v>1.79</v>
+      </c>
+      <c r="I287" s="5">
+        <v>1.8</v>
+      </c>
+      <c r="J287" s="5">
+        <v>1.79</v>
+      </c>
+      <c r="K287" s="5">
+        <v>1.86</v>
+      </c>
+      <c r="L287" s="5">
+        <v>2.21</v>
+      </c>
+      <c r="M287" s="5">
+        <v>1.99</v>
+      </c>
+      <c r="N287" s="5">
+        <v>1.88</v>
+      </c>
+      <c r="O287" s="5">
+        <v>2</v>
+      </c>
+      <c r="P287" s="5">
+        <v>1.96</v>
+      </c>
+      <c r="Q287" s="5">
+        <v>2.21</v>
+      </c>
+      <c r="R287" s="5">
+        <v>2.19</v>
+      </c>
+      <c r="S287" s="5">
+        <v>2.21</v>
+      </c>
+      <c r="T287" s="5">
+        <v>3.27</v>
+      </c>
+      <c r="U287" s="5">
+        <v>4.07</v>
+      </c>
+      <c r="V287" s="3"/>
       <c r="W287" s="2" t="s">
-        <v>30</v>
+        <v>400</v>
       </c>
     </row>
     <row r="288" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A288" s="2" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>391</v>
+        <v>401</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>393</v>
+        <v>402</v>
       </c>
       <c r="D288" s="2" t="s">
-        <v>90</v>
+        <v>27</v>
       </c>
       <c r="E288" s="3" t="s">
-        <v>399</v>
+        <v>28</v>
       </c>
       <c r="F288" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G288" s="4">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="H288" s="4">
-        <v>5</v>
-      </c>
-      <c r="I288" s="4">
-        <v>6.8</v>
-      </c>
-      <c r="J288" s="4">
-        <v>3.7</v>
-      </c>
-      <c r="K288" s="4">
-        <v>6.6</v>
-      </c>
-      <c r="L288" s="4">
-        <v>6</v>
-      </c>
-      <c r="M288" s="4">
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="N288" s="4">
-        <v>8.4</v>
-      </c>
-      <c r="O288" s="4">
-        <v>10.9</v>
-      </c>
-      <c r="P288" s="4">
-        <v>12.2</v>
-      </c>
-      <c r="Q288" s="4">
-        <v>13.5</v>
-      </c>
-      <c r="R288" s="4">
-        <v>15.8</v>
-      </c>
-      <c r="S288" s="4">
-        <v>23.6</v>
-      </c>
-      <c r="T288" s="4">
-        <v>26.1</v>
-      </c>
+      <c r="G288" s="3"/>
+      <c r="H288" s="3"/>
+      <c r="I288" s="3"/>
+      <c r="J288" s="3"/>
+      <c r="K288" s="3"/>
+      <c r="L288" s="3"/>
+      <c r="M288" s="3"/>
+      <c r="N288" s="3"/>
+      <c r="O288" s="3"/>
+      <c r="P288" s="3"/>
+      <c r="Q288" s="3"/>
+      <c r="R288" s="3"/>
+      <c r="S288" s="3"/>
+      <c r="T288" s="3"/>
       <c r="U288" s="4">
-        <v>27.4</v>
+        <v>30.2</v>
       </c>
       <c r="V288" s="4">
-        <v>27.6</v>
+        <v>51.3</v>
       </c>
       <c r="W288" s="2" t="s">
         <v>30</v>
@@ -20007,16 +20009,16 @@
     </row>
     <row r="289" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A289" s="2" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="D289" s="2" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="E289" s="3" t="s">
         <v>28</v>
@@ -20025,454 +20027,492 @@
         <v>34</v>
       </c>
       <c r="G289" s="4">
-        <v>5.7</v>
+        <v>28.1</v>
       </c>
       <c r="H289" s="4">
-        <v>6</v>
+        <v>27.6</v>
       </c>
       <c r="I289" s="4">
-        <v>4.9000000000000004</v>
+        <v>31.6</v>
       </c>
       <c r="J289" s="4">
-        <v>4.3</v>
+        <v>22.6</v>
       </c>
       <c r="K289" s="4">
-        <v>4.7</v>
+        <v>26.9</v>
       </c>
       <c r="L289" s="4">
-        <v>4.5</v>
+        <v>26.6</v>
       </c>
       <c r="M289" s="4">
-        <v>3.3</v>
+        <v>30.2</v>
       </c>
       <c r="N289" s="4">
-        <v>3.8</v>
+        <v>30.8</v>
       </c>
       <c r="O289" s="4">
-        <v>4.5999999999999996</v>
+        <v>35.5</v>
       </c>
       <c r="P289" s="4">
-        <v>4.3</v>
+        <v>40.4</v>
       </c>
       <c r="Q289" s="4">
-        <v>4.4000000000000004</v>
+        <v>41.9</v>
       </c>
       <c r="R289" s="4">
-        <v>4.0999999999999996</v>
+        <v>47.5</v>
       </c>
       <c r="S289" s="4">
-        <v>3.8</v>
+        <v>55.4</v>
       </c>
       <c r="T289" s="4">
-        <v>5.0999999999999996</v>
+        <v>58.5</v>
       </c>
       <c r="U289" s="4">
-        <v>4.8</v>
+        <v>61</v>
       </c>
       <c r="V289" s="4">
-        <v>5.2</v>
+        <v>61.1</v>
       </c>
       <c r="W289" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="290" spans="1:23" ht="45" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A290" s="2" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C290" s="2" t="s">
         <v>403</v>
       </c>
       <c r="D290" s="2" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="E290" s="3" t="s">
-        <v>28</v>
+        <v>404</v>
       </c>
       <c r="F290" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G290" s="6">
-        <v>674</v>
-      </c>
-      <c r="H290" s="6">
-        <v>605</v>
-      </c>
-      <c r="I290" s="6">
-        <v>1082</v>
-      </c>
-      <c r="J290" s="6">
-        <v>1219</v>
-      </c>
-      <c r="K290" s="6">
-        <v>1282</v>
-      </c>
-      <c r="L290" s="6">
-        <v>1456</v>
-      </c>
-      <c r="M290" s="6">
-        <v>1926</v>
-      </c>
-      <c r="N290" s="6">
-        <v>3182</v>
-      </c>
-      <c r="O290" s="6">
-        <v>3739</v>
-      </c>
-      <c r="P290" s="6">
-        <v>6484</v>
-      </c>
-      <c r="Q290" s="6">
-        <v>10420</v>
-      </c>
-      <c r="R290" s="6">
-        <v>29483</v>
-      </c>
-      <c r="S290" s="6">
-        <v>39683</v>
-      </c>
-      <c r="T290" s="6">
-        <v>80267</v>
-      </c>
-      <c r="U290" s="6">
-        <v>103449</v>
-      </c>
-      <c r="V290" s="6">
-        <v>260783</v>
+        <v>34</v>
+      </c>
+      <c r="G290" s="4">
+        <v>31.5</v>
+      </c>
+      <c r="H290" s="4">
+        <v>27.9</v>
+      </c>
+      <c r="I290" s="4">
+        <v>36.799999999999997</v>
+      </c>
+      <c r="J290" s="4">
+        <v>20.2</v>
+      </c>
+      <c r="K290" s="4">
+        <v>23.9</v>
+      </c>
+      <c r="L290" s="4">
+        <v>20.8</v>
+      </c>
+      <c r="M290" s="4">
+        <v>20.5</v>
+      </c>
+      <c r="N290" s="4">
+        <v>22.4</v>
+      </c>
+      <c r="O290" s="4">
+        <v>29.5</v>
+      </c>
+      <c r="P290" s="4">
+        <v>29.8</v>
+      </c>
+      <c r="Q290" s="4">
+        <v>30.9</v>
+      </c>
+      <c r="R290" s="4">
+        <v>35.6</v>
+      </c>
+      <c r="S290" s="4">
+        <v>42.1</v>
+      </c>
+      <c r="T290" s="4">
+        <v>44</v>
+      </c>
+      <c r="U290" s="4">
+        <v>47.7</v>
+      </c>
+      <c r="V290" s="4">
+        <v>48.9</v>
       </c>
       <c r="W290" s="2" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="291" spans="1:23" ht="45" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="291" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A291" s="2" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C291" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="D291" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E291" s="3" t="s">
         <v>405</v>
-      </c>
-      <c r="D291" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E291" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="F291" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G291" s="3"/>
-      <c r="H291" s="3"/>
-      <c r="I291" s="3"/>
-      <c r="J291" s="3"/>
-      <c r="K291" s="3"/>
-      <c r="L291" s="3"/>
-      <c r="M291" s="3"/>
-      <c r="N291" s="3"/>
-      <c r="O291" s="3"/>
-      <c r="P291" s="3"/>
-      <c r="Q291" s="3"/>
-      <c r="R291" s="5">
-        <v>18.93</v>
-      </c>
-      <c r="S291" s="3"/>
-      <c r="T291" s="5">
-        <v>21.3</v>
-      </c>
-      <c r="U291" s="3"/>
-      <c r="V291" s="5">
-        <v>23.01</v>
+      <c r="G291" s="4">
+        <v>47.6</v>
+      </c>
+      <c r="H291" s="4">
+        <v>46.2</v>
+      </c>
+      <c r="I291" s="4">
+        <v>50.6</v>
+      </c>
+      <c r="J291" s="4">
+        <v>39</v>
+      </c>
+      <c r="K291" s="4">
+        <v>46</v>
+      </c>
+      <c r="L291" s="4">
+        <v>45</v>
+      </c>
+      <c r="M291" s="4">
+        <v>48.1</v>
+      </c>
+      <c r="N291" s="4">
+        <v>48.1</v>
+      </c>
+      <c r="O291" s="4">
+        <v>53</v>
+      </c>
+      <c r="P291" s="4">
+        <v>58.6</v>
+      </c>
+      <c r="Q291" s="4">
+        <v>59.9</v>
+      </c>
+      <c r="R291" s="4">
+        <v>68.3</v>
+      </c>
+      <c r="S291" s="4">
+        <v>75.2</v>
+      </c>
+      <c r="T291" s="4">
+        <v>81</v>
+      </c>
+      <c r="U291" s="4">
+        <v>81.2</v>
+      </c>
+      <c r="V291" s="4">
+        <v>81.8</v>
       </c>
       <c r="W291" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="292" spans="1:23" ht="36" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="292" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A292" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="B292" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="C292" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="D292" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E292" s="3" t="s">
         <v>406</v>
       </c>
-      <c r="B292" s="2" t="s">
+      <c r="F292" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G292" s="4">
+        <v>37.6</v>
+      </c>
+      <c r="H292" s="4">
+        <v>36.9</v>
+      </c>
+      <c r="I292" s="4">
+        <v>45.3</v>
+      </c>
+      <c r="J292" s="4">
+        <v>35.200000000000003</v>
+      </c>
+      <c r="K292" s="4">
+        <v>40.1</v>
+      </c>
+      <c r="L292" s="4">
+        <v>38.6</v>
+      </c>
+      <c r="M292" s="4">
+        <v>40.5</v>
+      </c>
+      <c r="N292" s="4">
+        <v>45</v>
+      </c>
+      <c r="O292" s="4">
+        <v>49.6</v>
+      </c>
+      <c r="P292" s="4">
+        <v>57.6</v>
+      </c>
+      <c r="Q292" s="4">
+        <v>59.4</v>
+      </c>
+      <c r="R292" s="4">
+        <v>65.900000000000006</v>
+      </c>
+      <c r="S292" s="4">
+        <v>75.599999999999994</v>
+      </c>
+      <c r="T292" s="4">
+        <v>78.3</v>
+      </c>
+      <c r="U292" s="4">
+        <v>81.099999999999994</v>
+      </c>
+      <c r="V292" s="4">
+        <v>78.3</v>
+      </c>
+      <c r="W292" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="293" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+      <c r="A293" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="B293" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="C293" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="D293" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E293" s="3" t="s">
         <v>407</v>
       </c>
-      <c r="C292" s="2" t="s">
+      <c r="F293" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G293" s="4">
+        <v>26.2</v>
+      </c>
+      <c r="H293" s="4">
+        <v>26.3</v>
+      </c>
+      <c r="I293" s="4">
+        <v>28.7</v>
+      </c>
+      <c r="J293" s="4">
+        <v>21.5</v>
+      </c>
+      <c r="K293" s="4">
+        <v>26.2</v>
+      </c>
+      <c r="L293" s="4">
+        <v>26</v>
+      </c>
+      <c r="M293" s="4">
+        <v>30</v>
+      </c>
+      <c r="N293" s="4">
+        <v>28</v>
+      </c>
+      <c r="O293" s="4">
+        <v>35</v>
+      </c>
+      <c r="P293" s="4">
+        <v>41.4</v>
+      </c>
+      <c r="Q293" s="4">
+        <v>45.1</v>
+      </c>
+      <c r="R293" s="4">
+        <v>51.7</v>
+      </c>
+      <c r="S293" s="4">
+        <v>62.4</v>
+      </c>
+      <c r="T293" s="4">
+        <v>65.7</v>
+      </c>
+      <c r="U293" s="4">
+        <v>68.8</v>
+      </c>
+      <c r="V293" s="4">
+        <v>69.900000000000006</v>
+      </c>
+      <c r="W293" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="294" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+      <c r="A294" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="B294" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="C294" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="D294" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E294" s="3" t="s">
         <v>408</v>
-      </c>
-      <c r="D292" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E292" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F292" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="G292" s="5">
-        <v>377.75</v>
-      </c>
-      <c r="H292" s="5">
-        <v>417.47</v>
-      </c>
-      <c r="I292" s="5">
-        <v>421.06</v>
-      </c>
-      <c r="J292" s="5">
-        <v>487.12</v>
-      </c>
-      <c r="K292" s="5">
-        <v>451.84</v>
-      </c>
-      <c r="L292" s="5">
-        <v>440.89</v>
-      </c>
-      <c r="M292" s="5">
-        <v>662.95</v>
-      </c>
-      <c r="N292" s="5">
-        <v>679.46</v>
-      </c>
-      <c r="O292" s="5">
-        <v>766.04</v>
-      </c>
-      <c r="P292" s="5">
-        <v>776.56</v>
-      </c>
-      <c r="Q292" s="5">
-        <v>829.27</v>
-      </c>
-      <c r="R292" s="5">
-        <v>983.51</v>
-      </c>
-      <c r="S292" s="5">
-        <v>3494.39</v>
-      </c>
-      <c r="T292" s="5">
-        <v>2580.38</v>
-      </c>
-      <c r="U292" s="5">
-        <v>1840.15</v>
-      </c>
-      <c r="V292" s="3"/>
-      <c r="W292" s="2" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="293" spans="1:23" ht="36" x14ac:dyDescent="0.25">
-      <c r="A293" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="B293" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="C293" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="D293" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E293" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F293" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="G293" s="5">
-        <v>96.04</v>
-      </c>
-      <c r="H293" s="5">
-        <v>90.68</v>
-      </c>
-      <c r="I293" s="5">
-        <v>111.55</v>
-      </c>
-      <c r="J293" s="5">
-        <v>127.11</v>
-      </c>
-      <c r="K293" s="5">
-        <v>82.28</v>
-      </c>
-      <c r="L293" s="5">
-        <v>100.19</v>
-      </c>
-      <c r="M293" s="5">
-        <v>148.99</v>
-      </c>
-      <c r="N293" s="5">
-        <v>222.11</v>
-      </c>
-      <c r="O293" s="5">
-        <v>244.93</v>
-      </c>
-      <c r="P293" s="5">
-        <v>223.31</v>
-      </c>
-      <c r="Q293" s="5">
-        <v>225.08</v>
-      </c>
-      <c r="R293" s="5">
-        <v>296.20999999999998</v>
-      </c>
-      <c r="S293" s="5">
-        <v>2661.32</v>
-      </c>
-      <c r="T293" s="5">
-        <v>1701.94</v>
-      </c>
-      <c r="U293" s="5">
-        <v>705.25</v>
-      </c>
-      <c r="V293" s="3"/>
-      <c r="W293" s="2" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="294" spans="1:23" ht="72" x14ac:dyDescent="0.25">
-      <c r="A294" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="B294" s="2" t="s">
-        <v>413</v>
-      </c>
-      <c r="C294" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="D294" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E294" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="F294" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G294" s="5">
-        <v>0.08</v>
-      </c>
-      <c r="H294" s="5">
-        <v>0.08</v>
-      </c>
-      <c r="I294" s="5">
-        <v>0.09</v>
-      </c>
-      <c r="J294" s="5">
-        <v>0.1</v>
-      </c>
-      <c r="K294" s="5">
-        <v>0.09</v>
-      </c>
-      <c r="L294" s="5">
-        <v>0.1</v>
-      </c>
-      <c r="M294" s="5">
-        <v>0.15</v>
-      </c>
-      <c r="N294" s="5">
-        <v>0.13</v>
-      </c>
-      <c r="O294" s="5">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="P294" s="5">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="Q294" s="5">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="R294" s="5">
-        <v>0.15</v>
-      </c>
-      <c r="S294" s="5">
-        <v>0.53</v>
-      </c>
-      <c r="T294" s="5">
-        <v>0.33</v>
-      </c>
-      <c r="U294" s="5">
-        <v>0.21</v>
-      </c>
-      <c r="V294" s="3"/>
+      <c r="G294" s="4">
+        <v>13.5</v>
+      </c>
+      <c r="H294" s="4">
+        <v>15.7</v>
+      </c>
+      <c r="I294" s="4">
+        <v>17.2</v>
+      </c>
+      <c r="J294" s="4">
+        <v>12.7</v>
+      </c>
+      <c r="K294" s="4">
+        <v>15.5</v>
+      </c>
+      <c r="L294" s="4">
+        <v>18.3</v>
+      </c>
+      <c r="M294" s="4">
+        <v>19.8</v>
+      </c>
+      <c r="N294" s="4">
+        <v>18.8</v>
+      </c>
+      <c r="O294" s="4">
+        <v>22.4</v>
+      </c>
+      <c r="P294" s="4">
+        <v>28.5</v>
+      </c>
+      <c r="Q294" s="4">
+        <v>29.4</v>
+      </c>
+      <c r="R294" s="4">
+        <v>35</v>
+      </c>
+      <c r="S294" s="4">
+        <v>39.5</v>
+      </c>
+      <c r="T294" s="4">
+        <v>44.4</v>
+      </c>
+      <c r="U294" s="4">
+        <v>50.8</v>
+      </c>
+      <c r="V294" s="4">
+        <v>51.4</v>
+      </c>
       <c r="W294" s="2" t="s">
-        <v>410</v>
+        <v>30</v>
       </c>
     </row>
     <row r="295" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A295" s="2" t="s">
-        <v>406</v>
+        <v>390</v>
       </c>
       <c r="B295" s="2" t="s">
-        <v>415</v>
+        <v>401</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>416</v>
+        <v>403</v>
       </c>
       <c r="D295" s="2" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="E295" s="3" t="s">
-        <v>28</v>
+        <v>409</v>
       </c>
       <c r="F295" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="G295" s="3"/>
-      <c r="H295" s="3"/>
-      <c r="I295" s="3"/>
-      <c r="J295" s="7">
-        <v>2.2850000000000001</v>
-      </c>
-      <c r="K295" s="7">
-        <v>1.1160000000000001</v>
-      </c>
-      <c r="L295" s="7">
-        <v>1.55</v>
-      </c>
-      <c r="M295" s="7">
-        <v>3.7469999999999999</v>
-      </c>
-      <c r="N295" s="7">
-        <v>3.8530000000000002</v>
-      </c>
-      <c r="O295" s="7">
-        <v>3.367</v>
-      </c>
-      <c r="P295" s="7">
-        <v>6.8940000000000001</v>
-      </c>
-      <c r="Q295" s="7">
-        <v>4.077</v>
-      </c>
-      <c r="R295" s="7">
-        <v>4.49</v>
-      </c>
-      <c r="S295" s="7">
-        <v>11.999000000000001</v>
-      </c>
-      <c r="T295" s="7">
-        <v>16.606000000000002</v>
-      </c>
-      <c r="U295" s="7">
-        <v>20.382000000000001</v>
-      </c>
-      <c r="V295" s="7">
-        <v>5.3920000000000003</v>
+        <v>34</v>
+      </c>
+      <c r="G295" s="4">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="H295" s="4">
+        <v>5</v>
+      </c>
+      <c r="I295" s="4">
+        <v>6.8</v>
+      </c>
+      <c r="J295" s="4">
+        <v>3.7</v>
+      </c>
+      <c r="K295" s="4">
+        <v>6.6</v>
+      </c>
+      <c r="L295" s="4">
+        <v>6</v>
+      </c>
+      <c r="M295" s="4">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="N295" s="4">
+        <v>8.4</v>
+      </c>
+      <c r="O295" s="4">
+        <v>10.9</v>
+      </c>
+      <c r="P295" s="4">
+        <v>12.2</v>
+      </c>
+      <c r="Q295" s="4">
+        <v>13.5</v>
+      </c>
+      <c r="R295" s="4">
+        <v>15.8</v>
+      </c>
+      <c r="S295" s="4">
+        <v>23.6</v>
+      </c>
+      <c r="T295" s="4">
+        <v>26.1</v>
+      </c>
+      <c r="U295" s="4">
+        <v>27.4</v>
+      </c>
+      <c r="V295" s="4">
+        <v>27.6</v>
       </c>
       <c r="W295" s="2" t="s">
-        <v>417</v>
+        <v>30</v>
       </c>
     </row>
     <row r="296" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A296" s="2" t="s">
-        <v>406</v>
+        <v>390</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="D296" s="2" t="s">
         <v>27</v>
@@ -20481,61 +20521,69 @@
         <v>28</v>
       </c>
       <c r="F296" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="G296" s="3"/>
-      <c r="H296" s="3"/>
-      <c r="I296" s="3"/>
-      <c r="J296" s="5">
-        <v>8.07</v>
-      </c>
-      <c r="K296" s="5">
-        <v>3.54</v>
-      </c>
-      <c r="L296" s="5">
-        <v>2.98</v>
-      </c>
-      <c r="M296" s="5">
-        <v>2.44</v>
-      </c>
-      <c r="N296" s="5">
-        <v>2.25</v>
-      </c>
-      <c r="O296" s="5">
-        <v>63.36</v>
-      </c>
-      <c r="P296" s="5">
-        <v>7.61</v>
-      </c>
-      <c r="Q296" s="5">
-        <v>6.64</v>
-      </c>
-      <c r="R296" s="5">
-        <v>3.65</v>
-      </c>
-      <c r="S296" s="5">
-        <v>9.59</v>
-      </c>
-      <c r="T296" s="5">
-        <v>4.2699999999999996</v>
-      </c>
-      <c r="U296" s="5">
-        <v>8.32</v>
-      </c>
-      <c r="V296" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="G296" s="4">
+        <v>5.7</v>
+      </c>
+      <c r="H296" s="4">
+        <v>6</v>
+      </c>
+      <c r="I296" s="4">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="J296" s="4">
+        <v>4.3</v>
+      </c>
+      <c r="K296" s="4">
+        <v>4.7</v>
+      </c>
+      <c r="L296" s="4">
+        <v>4.5</v>
+      </c>
+      <c r="M296" s="4">
+        <v>3.3</v>
+      </c>
+      <c r="N296" s="4">
+        <v>3.8</v>
+      </c>
+      <c r="O296" s="4">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="P296" s="4">
+        <v>4.3</v>
+      </c>
+      <c r="Q296" s="4">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="R296" s="4">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="S296" s="4">
+        <v>3.8</v>
+      </c>
+      <c r="T296" s="4">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="U296" s="4">
+        <v>4.8</v>
+      </c>
+      <c r="V296" s="4">
+        <v>5.2</v>
+      </c>
       <c r="W296" s="2" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="297" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="297" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A297" s="2" t="s">
-        <v>406</v>
+        <v>390</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>419</v>
+        <v>412</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="D297" s="2" t="s">
         <v>27</v>
@@ -20544,55 +20592,69 @@
         <v>28</v>
       </c>
       <c r="F297" s="3" t="s">
-        <v>421</v>
-      </c>
-      <c r="G297" s="3"/>
-      <c r="H297" s="3"/>
-      <c r="I297" s="3"/>
-      <c r="J297" s="3"/>
+        <v>42</v>
+      </c>
+      <c r="G297" s="6">
+        <v>674</v>
+      </c>
+      <c r="H297" s="6">
+        <v>605</v>
+      </c>
+      <c r="I297" s="6">
+        <v>1082</v>
+      </c>
+      <c r="J297" s="6">
+        <v>1219</v>
+      </c>
       <c r="K297" s="6">
-        <v>1</v>
+        <v>1282</v>
       </c>
       <c r="L297" s="6">
-        <v>1</v>
+        <v>1456</v>
       </c>
       <c r="M297" s="6">
-        <v>8</v>
+        <v>1926</v>
       </c>
       <c r="N297" s="6">
-        <v>2</v>
-      </c>
-      <c r="O297" s="3"/>
+        <v>3182</v>
+      </c>
+      <c r="O297" s="6">
+        <v>3739</v>
+      </c>
       <c r="P297" s="6">
-        <v>1</v>
+        <v>6484</v>
       </c>
       <c r="Q297" s="6">
-        <v>2</v>
-      </c>
-      <c r="R297" s="3"/>
-      <c r="S297" s="3"/>
+        <v>10420</v>
+      </c>
+      <c r="R297" s="6">
+        <v>29483</v>
+      </c>
+      <c r="S297" s="6">
+        <v>39683</v>
+      </c>
       <c r="T297" s="6">
-        <v>8</v>
+        <v>80267</v>
       </c>
       <c r="U297" s="6">
-        <v>7</v>
+        <v>103449</v>
       </c>
       <c r="V297" s="6">
-        <v>2</v>
+        <v>260783</v>
       </c>
       <c r="W297" s="2" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="298" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="298" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A298" s="2" t="s">
-        <v>406</v>
+        <v>390</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>423</v>
+        <v>412</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>424</v>
+        <v>415</v>
       </c>
       <c r="D298" s="2" t="s">
         <v>27</v>
@@ -20601,65 +20663,43 @@
         <v>28</v>
       </c>
       <c r="F298" s="3" t="s">
-        <v>421</v>
+        <v>34</v>
       </c>
       <c r="G298" s="3"/>
       <c r="H298" s="3"/>
-      <c r="I298" s="6">
-        <v>2</v>
-      </c>
-      <c r="J298" s="6">
-        <v>2</v>
-      </c>
-      <c r="K298" s="6">
-        <v>1</v>
-      </c>
-      <c r="L298" s="6">
-        <v>1</v>
-      </c>
-      <c r="M298" s="6">
-        <v>1</v>
-      </c>
-      <c r="N298" s="6">
-        <v>1</v>
-      </c>
-      <c r="O298" s="6">
-        <v>1</v>
-      </c>
-      <c r="P298" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q298" s="6">
-        <v>4</v>
-      </c>
-      <c r="R298" s="6">
-        <v>1</v>
-      </c>
-      <c r="S298" s="6">
-        <v>1</v>
-      </c>
-      <c r="T298" s="6">
-        <v>0</v>
-      </c>
-      <c r="U298" s="6">
-        <v>4</v>
-      </c>
-      <c r="V298" s="6">
-        <v>2</v>
+      <c r="I298" s="3"/>
+      <c r="J298" s="3"/>
+      <c r="K298" s="3"/>
+      <c r="L298" s="3"/>
+      <c r="M298" s="3"/>
+      <c r="N298" s="3"/>
+      <c r="O298" s="3"/>
+      <c r="P298" s="3"/>
+      <c r="Q298" s="3"/>
+      <c r="R298" s="5">
+        <v>18.93</v>
+      </c>
+      <c r="S298" s="3"/>
+      <c r="T298" s="5">
+        <v>21.3</v>
+      </c>
+      <c r="U298" s="3"/>
+      <c r="V298" s="5">
+        <v>23.01</v>
       </c>
       <c r="W298" s="2" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="299" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="299" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A299" s="2" t="s">
-        <v>406</v>
+        <v>416</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="D299" s="2" t="s">
         <v>27</v>
@@ -20668,61 +20708,67 @@
         <v>28</v>
       </c>
       <c r="F299" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G299" s="3"/>
-      <c r="H299" s="3"/>
-      <c r="I299" s="3"/>
-      <c r="J299" s="3"/>
-      <c r="K299" s="6">
-        <v>5</v>
-      </c>
-      <c r="L299" s="6">
-        <v>13</v>
-      </c>
-      <c r="M299" s="6">
-        <v>19</v>
-      </c>
-      <c r="N299" s="6">
-        <v>18</v>
-      </c>
-      <c r="O299" s="6">
-        <v>15</v>
-      </c>
-      <c r="P299" s="6">
-        <v>15</v>
-      </c>
-      <c r="Q299" s="6">
-        <v>8</v>
-      </c>
-      <c r="R299" s="6">
-        <v>28</v>
-      </c>
-      <c r="S299" s="6">
-        <v>53</v>
-      </c>
-      <c r="T299" s="6">
-        <v>65</v>
-      </c>
-      <c r="U299" s="6">
-        <v>70</v>
-      </c>
-      <c r="V299" s="6">
-        <v>69</v>
-      </c>
+        <v>419</v>
+      </c>
+      <c r="G299" s="5">
+        <v>377.75</v>
+      </c>
+      <c r="H299" s="5">
+        <v>417.47</v>
+      </c>
+      <c r="I299" s="5">
+        <v>421.06</v>
+      </c>
+      <c r="J299" s="5">
+        <v>487.12</v>
+      </c>
+      <c r="K299" s="5">
+        <v>451.84</v>
+      </c>
+      <c r="L299" s="5">
+        <v>440.89</v>
+      </c>
+      <c r="M299" s="5">
+        <v>662.95</v>
+      </c>
+      <c r="N299" s="5">
+        <v>679.46</v>
+      </c>
+      <c r="O299" s="5">
+        <v>766.04</v>
+      </c>
+      <c r="P299" s="5">
+        <v>776.56</v>
+      </c>
+      <c r="Q299" s="5">
+        <v>829.27</v>
+      </c>
+      <c r="R299" s="5">
+        <v>983.51</v>
+      </c>
+      <c r="S299" s="5">
+        <v>3494.39</v>
+      </c>
+      <c r="T299" s="5">
+        <v>2580.38</v>
+      </c>
+      <c r="U299" s="5">
+        <v>1840.15</v>
+      </c>
+      <c r="V299" s="3"/>
       <c r="W299" s="2" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="300" spans="1:23" ht="36" x14ac:dyDescent="0.25">
+      <c r="A300" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B300" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="C300" s="2" t="s">
         <v>422</v>
-      </c>
-    </row>
-    <row r="300" spans="1:23" ht="45" x14ac:dyDescent="0.25">
-      <c r="A300" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="B300" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="C300" s="2" t="s">
-        <v>428</v>
       </c>
       <c r="D300" s="2" t="s">
         <v>27</v>
@@ -20731,47 +20777,500 @@
         <v>28</v>
       </c>
       <c r="F300" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="G300" s="5">
+        <v>96.04</v>
+      </c>
+      <c r="H300" s="5">
+        <v>90.68</v>
+      </c>
+      <c r="I300" s="5">
+        <v>111.55</v>
+      </c>
+      <c r="J300" s="5">
+        <v>127.11</v>
+      </c>
+      <c r="K300" s="5">
+        <v>82.28</v>
+      </c>
+      <c r="L300" s="5">
+        <v>100.19</v>
+      </c>
+      <c r="M300" s="5">
+        <v>148.99</v>
+      </c>
+      <c r="N300" s="5">
+        <v>222.11</v>
+      </c>
+      <c r="O300" s="5">
+        <v>244.93</v>
+      </c>
+      <c r="P300" s="5">
+        <v>223.31</v>
+      </c>
+      <c r="Q300" s="5">
+        <v>225.08</v>
+      </c>
+      <c r="R300" s="5">
+        <v>296.20999999999998</v>
+      </c>
+      <c r="S300" s="5">
+        <v>2661.32</v>
+      </c>
+      <c r="T300" s="5">
+        <v>1701.94</v>
+      </c>
+      <c r="U300" s="5">
+        <v>705.25</v>
+      </c>
+      <c r="V300" s="3"/>
+      <c r="W300" s="2" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="301" spans="1:23" ht="72" x14ac:dyDescent="0.25">
+      <c r="A301" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B301" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="C301" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="D301" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E301" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F301" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G301" s="5">
+        <v>0.08</v>
+      </c>
+      <c r="H301" s="5">
+        <v>0.08</v>
+      </c>
+      <c r="I301" s="5">
+        <v>0.09</v>
+      </c>
+      <c r="J301" s="5">
+        <v>0.1</v>
+      </c>
+      <c r="K301" s="5">
+        <v>0.09</v>
+      </c>
+      <c r="L301" s="5">
+        <v>0.1</v>
+      </c>
+      <c r="M301" s="5">
+        <v>0.15</v>
+      </c>
+      <c r="N301" s="5">
+        <v>0.13</v>
+      </c>
+      <c r="O301" s="5">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="P301" s="5">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="Q301" s="5">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="R301" s="5">
+        <v>0.15</v>
+      </c>
+      <c r="S301" s="5">
+        <v>0.53</v>
+      </c>
+      <c r="T301" s="5">
+        <v>0.33</v>
+      </c>
+      <c r="U301" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="V301" s="3"/>
+      <c r="W301" s="2" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="302" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+      <c r="A302" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B302" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="C302" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="D302" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E302" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F302" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="G302" s="3"/>
+      <c r="H302" s="3"/>
+      <c r="I302" s="3"/>
+      <c r="J302" s="7">
+        <v>2.2850000000000001</v>
+      </c>
+      <c r="K302" s="7">
+        <v>1.1160000000000001</v>
+      </c>
+      <c r="L302" s="7">
+        <v>1.55</v>
+      </c>
+      <c r="M302" s="7">
+        <v>3.7469999999999999</v>
+      </c>
+      <c r="N302" s="7">
+        <v>3.8530000000000002</v>
+      </c>
+      <c r="O302" s="7">
+        <v>3.367</v>
+      </c>
+      <c r="P302" s="7">
+        <v>6.8940000000000001</v>
+      </c>
+      <c r="Q302" s="7">
+        <v>4.077</v>
+      </c>
+      <c r="R302" s="7">
+        <v>4.49</v>
+      </c>
+      <c r="S302" s="7">
+        <v>11.999000000000001</v>
+      </c>
+      <c r="T302" s="7">
+        <v>16.606000000000002</v>
+      </c>
+      <c r="U302" s="7">
+        <v>20.382000000000001</v>
+      </c>
+      <c r="V302" s="7">
+        <v>5.3920000000000003</v>
+      </c>
+      <c r="W302" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="303" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+      <c r="A303" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B303" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="C303" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="D303" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E303" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F303" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="G303" s="3"/>
+      <c r="H303" s="3"/>
+      <c r="I303" s="3"/>
+      <c r="J303" s="5">
+        <v>8.07</v>
+      </c>
+      <c r="K303" s="5">
+        <v>3.54</v>
+      </c>
+      <c r="L303" s="5">
+        <v>2.98</v>
+      </c>
+      <c r="M303" s="5">
+        <v>2.44</v>
+      </c>
+      <c r="N303" s="5">
+        <v>2.25</v>
+      </c>
+      <c r="O303" s="5">
+        <v>63.36</v>
+      </c>
+      <c r="P303" s="5">
+        <v>7.61</v>
+      </c>
+      <c r="Q303" s="5">
+        <v>6.64</v>
+      </c>
+      <c r="R303" s="5">
+        <v>3.65</v>
+      </c>
+      <c r="S303" s="5">
+        <v>9.59</v>
+      </c>
+      <c r="T303" s="5">
+        <v>4.2699999999999996</v>
+      </c>
+      <c r="U303" s="5">
+        <v>8.32</v>
+      </c>
+      <c r="V303" s="3"/>
+      <c r="W303" s="2" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="304" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+      <c r="A304" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B304" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="C304" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="D304" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E304" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F304" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="G304" s="3"/>
+      <c r="H304" s="3"/>
+      <c r="I304" s="3"/>
+      <c r="J304" s="3"/>
+      <c r="K304" s="6">
+        <v>1</v>
+      </c>
+      <c r="L304" s="6">
+        <v>1</v>
+      </c>
+      <c r="M304" s="6">
+        <v>8</v>
+      </c>
+      <c r="N304" s="6">
+        <v>2</v>
+      </c>
+      <c r="O304" s="3"/>
+      <c r="P304" s="6">
+        <v>1</v>
+      </c>
+      <c r="Q304" s="6">
+        <v>2</v>
+      </c>
+      <c r="R304" s="3"/>
+      <c r="S304" s="3"/>
+      <c r="T304" s="6">
+        <v>8</v>
+      </c>
+      <c r="U304" s="6">
+        <v>7</v>
+      </c>
+      <c r="V304" s="6">
+        <v>2</v>
+      </c>
+      <c r="W304" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="305" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+      <c r="A305" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B305" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="C305" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="D305" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E305" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F305" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="G305" s="3"/>
+      <c r="H305" s="3"/>
+      <c r="I305" s="6">
+        <v>2</v>
+      </c>
+      <c r="J305" s="6">
+        <v>2</v>
+      </c>
+      <c r="K305" s="6">
+        <v>1</v>
+      </c>
+      <c r="L305" s="6">
+        <v>1</v>
+      </c>
+      <c r="M305" s="6">
+        <v>1</v>
+      </c>
+      <c r="N305" s="6">
+        <v>1</v>
+      </c>
+      <c r="O305" s="6">
+        <v>1</v>
+      </c>
+      <c r="P305" s="6">
+        <v>1</v>
+      </c>
+      <c r="Q305" s="6">
+        <v>4</v>
+      </c>
+      <c r="R305" s="6">
+        <v>1</v>
+      </c>
+      <c r="S305" s="6">
+        <v>1</v>
+      </c>
+      <c r="T305" s="6">
+        <v>0</v>
+      </c>
+      <c r="U305" s="6">
+        <v>4</v>
+      </c>
+      <c r="V305" s="6">
+        <v>2</v>
+      </c>
+      <c r="W305" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="306" spans="1:23" ht="27" x14ac:dyDescent="0.25">
+      <c r="A306" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B306" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="C306" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="D306" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E306" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F306" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G300" s="3"/>
-      <c r="H300" s="3"/>
-      <c r="I300" s="3"/>
-      <c r="J300" s="3"/>
-      <c r="K300" s="3"/>
-      <c r="L300" s="3"/>
-      <c r="M300" s="3"/>
-      <c r="N300" s="3"/>
-      <c r="O300" s="3"/>
-      <c r="P300" s="3"/>
-      <c r="Q300" s="3"/>
-      <c r="R300" s="3"/>
-      <c r="S300" s="3"/>
-      <c r="T300" s="6">
+      <c r="G306" s="3"/>
+      <c r="H306" s="3"/>
+      <c r="I306" s="3"/>
+      <c r="J306" s="3"/>
+      <c r="K306" s="6">
+        <v>5</v>
+      </c>
+      <c r="L306" s="6">
+        <v>13</v>
+      </c>
+      <c r="M306" s="6">
+        <v>19</v>
+      </c>
+      <c r="N306" s="6">
+        <v>18</v>
+      </c>
+      <c r="O306" s="6">
+        <v>15</v>
+      </c>
+      <c r="P306" s="6">
+        <v>15</v>
+      </c>
+      <c r="Q306" s="6">
+        <v>8</v>
+      </c>
+      <c r="R306" s="6">
+        <v>28</v>
+      </c>
+      <c r="S306" s="6">
+        <v>53</v>
+      </c>
+      <c r="T306" s="6">
+        <v>65</v>
+      </c>
+      <c r="U306" s="6">
+        <v>70</v>
+      </c>
+      <c r="V306" s="6">
+        <v>69</v>
+      </c>
+      <c r="W306" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="307" spans="1:23" ht="45" x14ac:dyDescent="0.25">
+      <c r="A307" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B307" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C307" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="D307" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E307" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F307" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G307" s="3"/>
+      <c r="H307" s="3"/>
+      <c r="I307" s="3"/>
+      <c r="J307" s="3"/>
+      <c r="K307" s="3"/>
+      <c r="L307" s="3"/>
+      <c r="M307" s="3"/>
+      <c r="N307" s="3"/>
+      <c r="O307" s="3"/>
+      <c r="P307" s="3"/>
+      <c r="Q307" s="3"/>
+      <c r="R307" s="3"/>
+      <c r="S307" s="3"/>
+      <c r="T307" s="6">
         <v>114</v>
       </c>
-      <c r="U300" s="6">
+      <c r="U307" s="6">
         <v>61</v>
       </c>
-      <c r="V300" s="6">
+      <c r="V307" s="6">
         <v>97</v>
       </c>
-      <c r="W300" s="2" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="301" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="302" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A302" s="10" t="s">
-        <v>430</v>
-      </c>
-      <c r="B302" s="8"/>
+      <c r="W307" s="2" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="308" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="309" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A309" s="10" t="s">
+        <v>440</v>
+      </c>
+      <c r="B309" s="8"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:C3" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A302:B302"/>
+    <mergeCell ref="A309:B309"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
Rewizja zestawu krajowego - poprawki 11.6.b i 10.2.b (Excel + PDF)
</commit_message>
<xml_diff>
--- a/assets/excel/en/national_sdg_indicators.xlsx
+++ b/assets/excel/en/national_sdg_indicators.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sidwab\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A037913B-D2A7-433F-86BC-9F6E5E42A691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC813D9E-950E-4268-BAE3-7577D0BB9491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1351,7 +1351,7 @@
     <t>The Ministry of Economic Development and Technology / The Chancellery of the  Prime Minister</t>
   </si>
   <si>
-    <t>Last update: 07-08-2026, 10:19</t>
+    <t>Last update: 07-08-2026, 12:58</t>
   </si>
 </sst>
 </file>
@@ -16266,49 +16266,49 @@
         <v>34</v>
       </c>
       <c r="G232" s="4">
-        <v>99.6</v>
+        <v>43.4</v>
       </c>
       <c r="H232" s="4">
-        <v>99.6</v>
+        <v>46.5</v>
       </c>
       <c r="I232" s="4">
-        <v>99.6</v>
+        <v>47.2</v>
       </c>
       <c r="J232" s="4">
-        <v>99.6</v>
+        <v>47.8</v>
       </c>
       <c r="K232" s="4">
-        <v>99.6</v>
+        <v>46.4</v>
       </c>
       <c r="L232" s="4">
-        <v>99.6</v>
+        <v>46.5</v>
       </c>
       <c r="M232" s="4">
-        <v>99.7</v>
+        <v>51.4</v>
       </c>
       <c r="N232" s="4">
-        <v>99.7</v>
+        <v>53.8</v>
       </c>
       <c r="O232" s="4">
-        <v>99.7</v>
+        <v>54</v>
       </c>
       <c r="P232" s="4">
-        <v>99.7</v>
+        <v>54.3</v>
       </c>
       <c r="Q232" s="4">
-        <v>99.8</v>
+        <v>58.5</v>
       </c>
       <c r="R232" s="4">
-        <v>99.8</v>
+        <v>61.4</v>
       </c>
       <c r="S232" s="4">
-        <v>99.8</v>
+        <v>60</v>
       </c>
       <c r="T232" s="4">
-        <v>99.8</v>
+        <v>62.3</v>
       </c>
       <c r="U232" s="4">
-        <v>99.8</v>
+        <v>59.6</v>
       </c>
       <c r="V232" s="3"/>
       <c r="W232" s="2" t="s">
@@ -16335,49 +16335,49 @@
         <v>34</v>
       </c>
       <c r="G233" s="4">
-        <v>43.4</v>
+        <v>99.6</v>
       </c>
       <c r="H233" s="4">
-        <v>46.5</v>
+        <v>99.6</v>
       </c>
       <c r="I233" s="4">
-        <v>47.2</v>
+        <v>99.6</v>
       </c>
       <c r="J233" s="4">
-        <v>47.8</v>
+        <v>99.6</v>
       </c>
       <c r="K233" s="4">
-        <v>46.4</v>
+        <v>99.6</v>
       </c>
       <c r="L233" s="4">
-        <v>46.5</v>
+        <v>99.6</v>
       </c>
       <c r="M233" s="4">
-        <v>51.4</v>
+        <v>99.7</v>
       </c>
       <c r="N233" s="4">
-        <v>53.8</v>
+        <v>99.7</v>
       </c>
       <c r="O233" s="4">
-        <v>54</v>
+        <v>99.7</v>
       </c>
       <c r="P233" s="4">
-        <v>54.3</v>
+        <v>99.7</v>
       </c>
       <c r="Q233" s="4">
-        <v>58.5</v>
+        <v>99.8</v>
       </c>
       <c r="R233" s="4">
-        <v>61.4</v>
+        <v>99.8</v>
       </c>
       <c r="S233" s="4">
-        <v>60</v>
+        <v>99.8</v>
       </c>
       <c r="T233" s="4">
-        <v>62.3</v>
+        <v>99.8</v>
       </c>
       <c r="U233" s="4">
-        <v>59.6</v>
+        <v>99.8</v>
       </c>
       <c r="V233" s="3"/>
       <c r="W233" s="2" t="s">

</xml_diff>